<commit_message>
chore(MB-T01,MB-T02): mark tasks done in tracker
</commit_message>
<xml_diff>
--- a/tracker/Meterbook_Tracker.xlsx
+++ b/tracker/Meterbook_Tracker.xlsx
@@ -739,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="B2:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -747,7 +747,6 @@
     <col width="100" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -5738,22 +5737,34 @@
       </c>
       <c r="K3" s="31" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="L3" s="32" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L3" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="M3" s="33">
         <f>IF(K3="Done",1,IF(L3="",0,MIN(1,L3)))</f>
         <v/>
       </c>
       <c r="N3" s="31" t="n"/>
-      <c r="O3" s="34" t="n"/>
+      <c r="O3" s="34" t="n">
+        <v>46318</v>
+      </c>
       <c r="P3" s="29">
         <f>IF(K3="Done",IF(O3="","Done",IF(J3="","Done",IF(O3&lt;=J3,"On time","Late"))),IF(K3="Blocked","BLOCKED",IF(I3="","",IF(TODAY()&gt;J3,"OVERDUE",IF(TODAY()&gt;=I3,"Active","Upcoming")))))</f>
         <v/>
       </c>
-      <c r="Q3" s="31" t="n"/>
-      <c r="R3" s="31" t="n"/>
+      <c r="Q3" s="31" t="inlineStr">
+        <is>
+          <t>commit 79c4389 (branch foundation)</t>
+        </is>
+      </c>
+      <c r="R3" s="31" t="inlineStr">
+        <is>
+          <t>CLAUDE.md, README, CONTRIBUTING, ADR-0000/0001, design + runbook templates, coding/testing/API/git standards</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="29" t="inlineStr">
@@ -5802,22 +5813,34 @@
       </c>
       <c r="K4" s="31" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="L4" s="32" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L4" s="32" t="n">
+        <v>1</v>
+      </c>
       <c r="M4" s="33">
         <f>IF(K4="Done",1,IF(L4="",0,MIN(1,L4)))</f>
         <v/>
       </c>
       <c r="N4" s="31" t="n"/>
-      <c r="O4" s="34" t="n"/>
+      <c r="O4" s="34" t="n">
+        <v>46318</v>
+      </c>
       <c r="P4" s="29">
         <f>IF(K4="Done",IF(O4="","Done",IF(J4="","Done",IF(O4&lt;=J4,"On time","Late"))),IF(K4="Blocked","BLOCKED",IF(I4="","",IF(TODAY()&gt;J4,"OVERDUE",IF(TODAY()&gt;=I4,"Active","Upcoming")))))</f>
         <v/>
       </c>
-      <c r="Q4" s="31" t="n"/>
-      <c r="R4" s="31" t="n"/>
+      <c r="Q4" s="31" t="inlineStr">
+        <is>
+          <t>commit 79c4389 (branch foundation)</t>
+        </is>
+      </c>
+      <c r="R4" s="31" t="inlineStr">
+        <is>
+          <t>docs/slo/template.md (burn-rate alerting) + docs/slo/error-budget-policy.md</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="29" t="inlineStr">

</xml_diff>

<commit_message>
chore(MB-T03): record progress in tracker
</commit_message>
<xml_diff>
--- a/tracker/Meterbook_Tracker.xlsx
+++ b/tracker/Meterbook_Tracker.xlsx
@@ -5865,7 +5865,7 @@
       </c>
       <c r="E5" s="29" t="inlineStr">
         <is>
-          <t>terraform plan/apply green from CI; state in S3 + DynamoDB lock</t>
+          <t>terraform plan/apply green from CI; state in S3 with native locking (ADR-0002)</t>
         </is>
       </c>
       <c r="F5" s="29" t="inlineStr">
@@ -5889,10 +5889,12 @@
       </c>
       <c r="K5" s="31" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="L5" s="32" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="L5" s="32" t="n">
+        <v>0.8</v>
+      </c>
       <c r="M5" s="33">
         <f>IF(K5="Done",1,IF(L5="",0,MIN(1,L5)))</f>
         <v/>
@@ -5903,8 +5905,16 @@
         <f>IF(K5="Done",IF(O5="","Done",IF(J5="","Done",IF(O5&lt;=J5,"On time","Late"))),IF(K5="Blocked","BLOCKED",IF(I5="","",IF(TODAY()&gt;J5,"OVERDUE",IF(TODAY()&gt;=I5,"Active","Upcoming")))))</f>
         <v/>
       </c>
-      <c r="Q5" s="31" t="n"/>
-      <c r="R5" s="31" t="n"/>
+      <c r="Q5" s="31" t="inlineStr">
+        <is>
+          <t>commit 1bea340 (branch mb-t03-terraform-baseline)</t>
+        </is>
+      </c>
+      <c r="R5" s="31" t="inlineStr">
+        <is>
+          <t>Done: modules, dev/prod envs, 37 terraform tests, fmt/validate/tflint/trivy clean. Remaining: first apply to AWS (needs an AWS account) and plan/apply from CI (MB-T05). DynamoDB lock replaced by S3-native locking per ADR-0002.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="29" t="inlineStr">

</xml_diff>

<commit_message>
chore(MB-T01,MB-T02,MB-T03): update evidence links in tracker
</commit_message>
<xml_diff>
--- a/tracker/Meterbook_Tracker.xlsx
+++ b/tracker/Meterbook_Tracker.xlsx
@@ -5757,12 +5757,12 @@
       </c>
       <c r="Q3" s="31" t="inlineStr">
         <is>
-          <t>commit 79c4389 (branch foundation)</t>
+          <t>commit 19024d4 (branch foundation)</t>
         </is>
       </c>
       <c r="R3" s="31" t="inlineStr">
         <is>
-          <t>CLAUDE.md, README, CONTRIBUTING, ADR-0000/0001, design + runbook templates, coding/testing/API/git standards</t>
+          <t>Engineering rules, README, CONTRIBUTING, ADR-0000/0001, design + runbook templates, coding/testing/API/git standards</t>
         </is>
       </c>
     </row>
@@ -5833,7 +5833,7 @@
       </c>
       <c r="Q4" s="31" t="inlineStr">
         <is>
-          <t>commit 79c4389 (branch foundation)</t>
+          <t>commit 19024d4 (branch foundation)</t>
         </is>
       </c>
       <c r="R4" s="31" t="inlineStr">
@@ -5907,7 +5907,7 @@
       </c>
       <c r="Q5" s="31" t="inlineStr">
         <is>
-          <t>commit 1bea340 (branch mb-t03-terraform-baseline)</t>
+          <t>commit 4d92693 (branch mb-t03-terraform-baseline)</t>
         </is>
       </c>
       <c r="R5" s="31" t="inlineStr">

</xml_diff>

<commit_message>
chore(MB-T05): record progress in tracker
</commit_message>
<xml_diff>
--- a/tracker/Meterbook_Tracker.xlsx
+++ b/tracker/Meterbook_Tracker.xlsx
@@ -6027,10 +6027,12 @@
       </c>
       <c r="K7" s="31" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="L7" s="32" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="L7" s="32" t="n">
+        <v>0.7</v>
+      </c>
       <c r="M7" s="33">
         <f>IF(K7="Done",1,IF(L7="",0,MIN(1,L7)))</f>
         <v/>
@@ -6041,8 +6043,16 @@
         <f>IF(K7="Done",IF(O7="","Done",IF(J7="","Done",IF(O7&lt;=J7,"On time","Late"))),IF(K7="Blocked","BLOCKED",IF(I7="","",IF(TODAY()&gt;J7,"OVERDUE",IF(TODAY()&gt;=I7,"Active","Upcoming")))))</f>
         <v/>
       </c>
-      <c r="Q7" s="31" t="n"/>
-      <c r="R7" s="31" t="n"/>
+      <c r="Q7" s="31" t="inlineStr">
+        <is>
+          <t>https://github.com/mhrj7/meterbook/pull/3</t>
+        </is>
+      </c>
+      <c r="R7" s="31" t="inlineStr">
+        <is>
+          <t>Done: ci.yml (Terraform checks, Gitleaks, actionlint, single ci check), reusable container.yml (Trivy gate, SBOM, cosign), Terraform plan/apply via OIDC, SHA-pinned actions, Dependabot, ADR-0003. Remaining: green CI run as evidence, pipeline time measured, CRITICAL-CVE gate exercised by the first service image.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="29" t="inlineStr">

</xml_diff>

<commit_message>
chore(MB-T05): record green CI run and pipeline time
</commit_message>
<xml_diff>
--- a/tracker/Meterbook_Tracker.xlsx
+++ b/tracker/Meterbook_Tracker.xlsx
@@ -6031,7 +6031,7 @@
         </is>
       </c>
       <c r="L7" s="32" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
       <c r="M7" s="33">
         <f>IF(K7="Done",1,IF(L7="",0,MIN(1,L7)))</f>
@@ -6045,12 +6045,12 @@
       </c>
       <c r="Q7" s="31" t="inlineStr">
         <is>
-          <t>https://github.com/mhrj7/meterbook/pull/3</t>
+          <t>https://github.com/mhrj7/meterbook/actions/runs/39905115436</t>
         </is>
       </c>
       <c r="R7" s="31" t="inlineStr">
         <is>
-          <t>Done: ci.yml (Terraform checks, Gitleaks, actionlint, single ci check), reusable container.yml (Trivy gate, SBOM, cosign), Terraform plan/apply via OIDC, SHA-pinned actions, Dependabot, ADR-0003. Remaining: green CI run as evidence, pipeline time measured, CRITICAL-CVE gate exercised by the first service image.</t>
+          <t>Green CI run on PR #3: 3.3 min wall clock (Terraform job 3.0 min). Done: ci.yml (Terraform fmt/validate/test/tflint/trivy, Gitleaks, actionlint, single ci check), reusable container.yml (Trivy CRITICAL gate, SBOM, cosign), Terraform plan/apply via OIDC, SHA-pinned actions, Dependabot, ADR-0003. Remaining: CRITICAL-CVE gate exercised by the first service image (MB-T07).</t>
         </is>
       </c>
     </row>
@@ -11585,13 +11585,23 @@
       </c>
       <c r="K9" s="31" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="L9" s="34" t="n"/>
-      <c r="M9" s="31" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="L9" s="34" t="n">
+        <v>46318</v>
+      </c>
+      <c r="M9" s="31" t="inlineStr">
+        <is>
+          <t>0 findings across full history</t>
+        </is>
+      </c>
       <c r="N9" s="31" t="n"/>
-      <c r="O9" s="31" t="n"/>
+      <c r="O9" s="31" t="inlineStr">
+        <is>
+          <t>https://github.com/mhrj7/meterbook/actions/runs/39905115436</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="29" t="inlineStr">
@@ -14195,7 +14205,9 @@
           <t>min</t>
         </is>
       </c>
-      <c r="H5" s="39" t="n"/>
+      <c r="H5" s="39" t="n">
+        <v>3.3</v>
+      </c>
       <c r="I5" s="29">
         <f>IF(H5="","PENDING",IF(E5="&lt;=",IF(H5&lt;=F5,"PASS","FAIL"),IF(H5&gt;=F5,"PASS","FAIL")))</f>
         <v/>
@@ -14205,10 +14217,24 @@
           <t>GitHub Actions</t>
         </is>
       </c>
-      <c r="K5" s="31" t="n"/>
-      <c r="L5" s="34" t="n"/>
-      <c r="M5" s="31" t="n"/>
-      <c r="N5" s="31" t="n"/>
+      <c r="K5" s="31" t="inlineStr">
+        <is>
+          <t>39905115436</t>
+        </is>
+      </c>
+      <c r="L5" s="34" t="n">
+        <v>46318</v>
+      </c>
+      <c r="M5" s="31" t="inlineStr">
+        <is>
+          <t>https://github.com/mhrj7/meterbook/actions/runs/39905115436</t>
+        </is>
+      </c>
+      <c r="N5" s="31" t="inlineStr">
+        <is>
+          <t>Wall clock from run created to last job completed, PR #3.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="29" t="inlineStr">

</xml_diff>

<commit_message>
chore(MB-T04): record progress in tracker
</commit_message>
<xml_diff>
--- a/tracker/Meterbook_Tracker.xlsx
+++ b/tracker/Meterbook_Tracker.xlsx
@@ -5963,10 +5963,12 @@
       </c>
       <c r="K6" s="31" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="L6" s="32" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="L6" s="32" t="n">
+        <v>0.8</v>
+      </c>
       <c r="M6" s="33">
         <f>IF(K6="Done",1,IF(L6="",0,MIN(1,L6)))</f>
         <v/>
@@ -5977,8 +5979,16 @@
         <f>IF(K6="Done",IF(O6="","Done",IF(J6="","Done",IF(O6&lt;=J6,"On time","Late"))),IF(K6="Blocked","BLOCKED",IF(I6="","",IF(TODAY()&gt;J6,"OVERDUE",IF(TODAY()&gt;=I6,"Active","Upcoming")))))</f>
         <v/>
       </c>
-      <c r="Q6" s="31" t="n"/>
-      <c r="R6" s="31" t="n"/>
+      <c r="Q6" s="31" t="inlineStr">
+        <is>
+          <t>https://github.com/mhrj7/meterbook/pull/4</t>
+        </is>
+      </c>
+      <c r="R6" s="31" t="inlineStr">
+        <is>
+          <t>Done: app-secrets module (KMS, empty shells, Pod Identity ESO role, exact-ARN policy), platform-secrets Helm chart, ADR-0004, runbook; 7 terraform + 18 chart tests; kind end-to-end test (runtime read, rotation, namespace isolation) in CI. Remaining: green e2e evidence, then real AWS once dev is applied and ESO is installed via ArgoCD (MB-T06).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">

</xml_diff>

<commit_message>
chore(MB-T03,MB-T04): record CI evidence and AWS progress in tracker
</commit_message>
<xml_diff>
--- a/tracker/Meterbook_Tracker.xlsx
+++ b/tracker/Meterbook_Tracker.xlsx
@@ -5893,7 +5893,7 @@
         </is>
       </c>
       <c r="L5" s="32" t="n">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
       <c r="M5" s="33">
         <f>IF(K5="Done",1,IF(L5="",0,MIN(1,L5)))</f>
@@ -5907,12 +5907,12 @@
       </c>
       <c r="Q5" s="31" t="inlineStr">
         <is>
-          <t>commit 4d92693 (branch mb-t03-terraform-baseline)</t>
+          <t>https://github.com/mhrj7/meterbook/pull/5</t>
         </is>
       </c>
       <c r="R5" s="31" t="inlineStr">
         <is>
-          <t>Done: modules, dev/prod envs, 37 terraform tests, fmt/validate/tflint/trivy clean. Remaining: first apply to AWS (needs an AWS account) and plan/apply from CI (MB-T05). DynamoDB lock replaced by S3-native locking per ADR-0002.</t>
+          <t>CI-owned bootstrap (state bucket, OIDC provider, plan/apply roles via import blocks), apply-verify-destroy workflow, verify-dev.sh (AWS API checks), DB subnets isolated from internet, eu-north-1. GitHub OIDC provider created in AWS. Remaining: apply role (needs owner approval), bootstrap + dev apply from CI (blocked until AWS finishes verifying the new account).</t>
         </is>
       </c>
     </row>
@@ -5967,7 +5967,7 @@
         </is>
       </c>
       <c r="L6" s="32" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="M6" s="33">
         <f>IF(K6="Done",1,IF(L6="",0,MIN(1,L6)))</f>
@@ -5981,12 +5981,12 @@
       </c>
       <c r="Q6" s="31" t="inlineStr">
         <is>
-          <t>https://github.com/mhrj7/meterbook/pull/4</t>
+          <t>https://github.com/mhrj7/meterbook/actions/runs/39912053895</t>
         </is>
       </c>
       <c r="R6" s="31" t="inlineStr">
         <is>
-          <t>Done: app-secrets module (KMS, empty shells, Pod Identity ESO role, exact-ARN policy), platform-secrets Helm chart, ADR-0004, runbook; 7 terraform + 18 chart tests; kind end-to-end test (runtime read, rotation, namespace isolation) in CI. Remaining: green e2e evidence, then real AWS once dev is applied and ESO is installed via ArgoCD (MB-T06).</t>
+          <t>Green CI incl. kind end-to-end (4/4: delivery, runtime read by a pod, rotation in 3s, namespace isolation) after fixing a false-green CI step and a moto crash. Remaining: verify on real AWS (secrets, ESO role, Pod Identity) once the AWS account finishes verification and dev is applied.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(MB-T03): record AWS setup progress in tracker
</commit_message>
<xml_diff>
--- a/tracker/Meterbook_Tracker.xlsx
+++ b/tracker/Meterbook_Tracker.xlsx
@@ -5907,12 +5907,12 @@
       </c>
       <c r="Q5" s="31" t="inlineStr">
         <is>
-          <t>https://github.com/mhrj7/meterbook/pull/5</t>
+          <t>https://github.com/mhrj7/meterbook/pull/7</t>
         </is>
       </c>
       <c r="R5" s="31" t="inlineStr">
         <is>
-          <t>CI-owned bootstrap (state bucket, OIDC provider, plan/apply roles via import blocks), apply-verify-destroy workflow, verify-dev.sh (AWS API checks), DB subnets isolated from internet, eu-north-1. GitHub OIDC provider created in AWS. Remaining: apply role (needs owner approval), bootstrap + dev apply from CI (blocked until AWS finishes verifying the new account).</t>
+          <t>In AWS (eu-north-1): GitHub OIDC provider and meterbook-terraform-apply role created; trust fixed to GitHub's immutable OIDC subjects after the first bootstrap run was rejected. GitHub environments dev/production limited to main. Stack merged to main (PRs #1-#6). Remaining: bootstrap run green (state bucket, plan role), then dev apply-verify-destroy once AWS finishes verifying the new account.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(MB-T03,MB-T04): mark done with real-AWS evidence
</commit_message>
<xml_diff>
--- a/tracker/Meterbook_Tracker.xlsx
+++ b/tracker/Meterbook_Tracker.xlsx
@@ -5889,30 +5889,32 @@
       </c>
       <c r="K5" s="31" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L5" s="32" t="n">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="M5" s="33">
         <f>IF(K5="Done",1,IF(L5="",0,MIN(1,L5)))</f>
         <v/>
       </c>
       <c r="N5" s="31" t="n"/>
-      <c r="O5" s="34" t="n"/>
+      <c r="O5" s="34" t="n">
+        <v>46318</v>
+      </c>
       <c r="P5" s="29">
         <f>IF(K5="Done",IF(O5="","Done",IF(J5="","Done",IF(O5&lt;=J5,"On time","Late"))),IF(K5="Blocked","BLOCKED",IF(I5="","",IF(TODAY()&gt;J5,"OVERDUE",IF(TODAY()&gt;=I5,"Active","Upcoming")))))</f>
         <v/>
       </c>
       <c r="Q5" s="31" t="inlineStr">
         <is>
-          <t>https://github.com/mhrj7/meterbook/pull/7</t>
+          <t>https://github.com/mhrj7/meterbook/actions/runs/39939409530</t>
         </is>
       </c>
       <c r="R5" s="31" t="inlineStr">
         <is>
-          <t>In AWS (eu-north-1): GitHub OIDC provider and meterbook-terraform-apply role created; trust fixed to GitHub's immutable OIDC subjects after the first bootstrap run was rejected. GitHub environments dev/production limited to main. Stack merged to main (PRs #1-#6). Remaining: bootstrap run green (state bucket, plan role), then dev apply-verify-destroy once AWS finishes verifying the new account.</t>
+          <t>Dev applied from CI on real AWS (eu-north-1): apply 12m54s, 35/35 baseline checks passed (state in S3 with native locking, EKS private+audited+KMS, nodes ACTIVE, RDS private/encrypted/TLS, buckets locked down, DB subnets without internet route), destroy removed 99 resources, 0 left. Fixed on the way: GitHub immutable OIDC subjects, Spot unavailable on new accounts, Free-plan instance types (dev uses m7i-flex.large), secrets recovery window on disposable envs.</t>
         </is>
       </c>
     </row>
@@ -5963,30 +5965,32 @@
       </c>
       <c r="K6" s="31" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L6" s="32" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="M6" s="33">
         <f>IF(K6="Done",1,IF(L6="",0,MIN(1,L6)))</f>
         <v/>
       </c>
       <c r="N6" s="31" t="n"/>
-      <c r="O6" s="34" t="n"/>
+      <c r="O6" s="34" t="n">
+        <v>46318</v>
+      </c>
       <c r="P6" s="29">
         <f>IF(K6="Done",IF(O6="","Done",IF(J6="","Done",IF(O6&lt;=J6,"On time","Late"))),IF(K6="Blocked","BLOCKED",IF(I6="","",IF(TODAY()&gt;J6,"OVERDUE",IF(TODAY()&gt;=I6,"Active","Upcoming")))))</f>
         <v/>
       </c>
       <c r="Q6" s="31" t="inlineStr">
         <is>
-          <t>https://github.com/mhrj7/meterbook/actions/runs/39912053895</t>
+          <t>https://github.com/mhrj7/meterbook/actions/runs/39939409530</t>
         </is>
       </c>
       <c r="R6" s="31" t="inlineStr">
         <is>
-          <t>Green CI incl. kind end-to-end (4/4: delivery, runtime read by a pod, rotation in 3s, namespace isolation) after fixing a false-green CI step and a moto crash. Remaining: verify on real AWS (secrets, ESO role, Pod Identity) once the AWS account finishes verification and dev is applied.</t>
+          <t>No secrets in git (Gitleaks, every run). Pods read secrets at runtime: kind end-to-end in CI (delivery, runtime read, rotation in 3s, namespace isolation; run 39912053895). On real AWS: 3 KMS-encrypted app secrets, ESO bound by Pod Identity, IAM simulation allows reading app secrets and denies other secrets and writes. ESO install on EKS follows with ArgoCD in MB-T06.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: evidence for the gap fixes; tracker test cases, coverage and CVE metric
TC-PLT-005 and TC-PLT-013 pass (SAST and linters), TC-PLT-006 updated (0
CRITICAL including unfixed), TC-PLT-020 (mTLS) and TC-PLT-021 (signed
images only) added and passing. Coverage rows for identity and tenancy
filled from CI (line, branch, mutation): both PASS. M-PLT-07 measured at 0.
EKS run 40117597732 passed 123/123.
</commit_message>
<xml_diff>
--- a/tracker/Meterbook_Tracker.xlsx
+++ b/tracker/Meterbook_Tracker.xlsx
@@ -163,7 +163,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1890" uniqueCount="1004">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1923" uniqueCount="1025">
   <si>
     <t xml:space="preserve">Meterbook — Plan, Test &amp; Reliability Tracker</t>
   </si>
@@ -735,7 +735,7 @@
     <t xml:space="preserve">https://github.com/mhrj7/meterbook/actions/runs/40006549728</t>
   </si>
   <si>
-    <t xml:space="preserve">First service image through the full pipeline on main (run 40006549728): Java tests gate the image; Trivy CRITICAL gate passed (0 fixable; 1 unfixed CRITICAL in the distroless Debian 13 base, libbrotli1 CVE-2026-111497, tracked until a patched base ships); SPDX SBOM; multi-arch push to GHCR; keyless cosign signature and SBOM attestation verified with cosign verify against the container.yml@refs/heads/main identity (and rejected for any other identity). PR pipeline: 3.3 min; image job 2m43s on PRs, 8m12s on main (multi-arch). Earlier: ci.yml, Terraform plan/apply via OIDC, SHA-pinned actions, Dependabot, ADR-0003.</t>
+    <t xml:space="preserve">First service image through the full pipeline on main (run 40006549728): Java tests gate the image; Trivy CRITICAL gate passed (0 fixable; 1 unfixed CRITICAL in the distroless Debian 13 base, libbrotli1 CVE-2026-111497, tracked until a patched base ships); SPDX SBOM; multi-arch push to GHCR; keyless cosign signature and SBOM attestation verified with cosign verify against the container.yml@refs/heads/main identity (and rejected for any other identity). PR pipeline: 3.3 min; image job 2m43s on PRs, 8m12s on main (multi-arch). Earlier: ci.yml, Terraform plan/apply via OIDC, SHA-pinned actions, Dependabot, ADR-0003. | 2026-10-25: SAST (CodeQL, Semgrep) and linters (SpotBugs, ruff, ShellCheck) added (TC-PLT-005/013); images also carry classic signatures for admission.</t>
   </si>
   <si>
     <t xml:space="preserve">MB-T06</t>
@@ -750,7 +750,7 @@
     <t xml:space="preserve">https://github.com/mhrj7/meterbook/actions/runs/39993278414</t>
   </si>
   <si>
-    <t xml:space="preserve">Real EKS dev cycle from main: apply 12m20s (101 resources), 60/60 checks passed in 4m05s, destroy 12m05s with 0 left. Terraform installs ArgoCD and one root per environment; ArgoCD deploys ESO, the secret store and the services ApplicationSet from Git. Secrets Manager values reach pods in meterbook-dev and meterbook-staging via Pod Identity; smoke service hardened; VPC CNI enforces NetworkPolicy. Every PR: ArgoCD on kind syncs dev+staging at the commit under test, 18/18 incl. staging self-heal (CI run 39991279763). Library chart with guard rails (38 render tests), GitOps policy check, prod pinned by SHA via scripts/promote-prod.sh, ADR-0006, runbook. Fixed on the way: podinfo command/args, ECR Public pull limits (Redis from mirror.gcr.io by digest), account ID masked in public logs. Evidence: docs/evidence/2026-10-23-dev-gitops-eks.md</t>
+    <t xml:space="preserve">Real EKS dev cycle from main: apply 12m20s (101 resources), 60/60 checks passed in 4m05s, destroy 12m05s with 0 left. Terraform installs ArgoCD and one root per environment; ArgoCD deploys ESO, the secret store and the services ApplicationSet from Git. Secrets Manager values reach pods in meterbook-dev and meterbook-staging via Pod Identity; smoke service hardened; VPC CNI enforces NetworkPolicy. Every PR: ArgoCD on kind syncs dev+staging at the commit under test, 18/18 incl. staging self-heal (CI run 39991279763). Library chart with guard rails (38 render tests), GitOps policy check, prod pinned by SHA via scripts/promote-prod.sh, ADR-0006, runbook. Fixed on the way: podinfo command/args, ECR Public pull limits (Redis from mirror.gcr.io by digest), account ID masked in public logs. Evidence: docs/evidence/2026-10-23-dev-gitops-eks.md | 2026-10-25: admission verifies signatures (ADR-0012, policy-controller); prod has identity, mesh, smoke and image policy, promoted; prod e2e on kind in CI.</t>
   </si>
   <si>
     <t xml:space="preserve">MB-T07</t>
@@ -768,7 +768,7 @@
     <t xml:space="preserve">https://github.com/mhrj7/meterbook/actions/runs/40065555690</t>
   </si>
   <si>
-    <t xml:space="preserve">DoD: SSO e2e in a real browser through a SAML IdP passes in CI on every identity change (TC-PLT-001; run 40065295770): tenant, SAML connection, SCIM token and user set up through the APIs; SSO sign-in lands in the tenant; JIT users join the tenant; another tenant's IdP asserting a victim's email is refused; SCIM deactivation kills the session and blocks sign-in. On EKS (run 40065555690): Keycloak + identity per environment via ArgoCD, db-bootstrap, operator creates a tenant, RDS isolation; 78/78 checks, 107 resources applied and destroyed. Built: ADR-0007/0008, design doc, OpenAPI contract with Spectral + oasdiff in CI, Spring Boot 4.1 on Java 25, Keycloak adapter, tenants, SAML SSO connections, SCIM 2.0 Users/Groups, Idempotency-Key, 158 tests (97% line / 87% branch). Found and fixed: cross-tenant account takeover via link-by-email; SCIM secret in idempotency store; Keycloak 26.8 domain routing; JIT onboarding; ArgoCD subchart dependency; a false-green CI pipeline (pipefail). Evidence: docs/evidence/2026-10-24-identity-sso-and-eks.md</t>
+    <t xml:space="preserve">DoD: SSO e2e in a real browser through a SAML IdP passes in CI on every identity change (TC-PLT-001; run 40065295770): tenant, SAML connection, SCIM token and user set up through the APIs; SSO sign-in lands in the tenant; JIT users join the tenant; another tenant's IdP asserting a victim's email is refused; SCIM deactivation kills the session and blocks sign-in. On EKS (run 40065555690): Keycloak + identity per environment via ArgoCD, db-bootstrap, operator creates a tenant, RDS isolation; 78/78 checks, 107 resources applied and destroyed. Built: ADR-0007/0008, design doc, OpenAPI contract with Spectral + oasdiff in CI, Spring Boot 4.1 on Java 25, Keycloak adapter, tenants, SAML SSO connections, SCIM 2.0 Users/Groups, Idempotency-Key, 158 tests (97% line / 87% branch). Found and fixed: cross-tenant account takeover via link-by-email; SCIM secret in idempotency store; Keycloak 26.8 domain routing; JIT onboarding; ArgoCD subchart dependency; a false-green CI pipeline (pipefail). Evidence: docs/evidence/2026-10-24-identity-sso-and-eks.md | 2026-10-25: Keycloak and identity run 2 replicas with PDBs in prod and dev; Keycloak clustering verified on EKS.</t>
   </si>
   <si>
     <t xml:space="preserve">MB-T08</t>
@@ -804,7 +804,7 @@
     <t xml:space="preserve">https://github.com/mhrj7/meterbook/actions/runs/40085243536</t>
   </si>
   <si>
-    <t xml:space="preserve">DoD: a revoked key is rejected on the very next request by identity (API test and browser e2e with a real Keycloak tenant admin, CI run 40084140187); other services may cache a verification for at most 30 s (Cache-Control: max-age=30; refusals no-store), so every service rejects it within 30 s. On EKS (run 40085243536): 87/87 checks, 107 resources applied and destroyed; /v1/api-key refuses no credentials, unknown keys and access tokens with no-store; V6 on RDS under forced RLS. Built: ADR-0010; keys mb_live_/mb_test_ + 238 random bits + CRC-32, SHA-256 at rest, shown once, never in idempotency records; one environment per key; scopes from a fixed vocabulary; expiry; rotation with a grace period; immediate revocation; 50 live keys per environment; last_used_at; keys cannot call the admin API. 193 tests (97.5% line / 87.1% branch). Found and fixed: timestamps serialised in the JVM zone instead of UTC; 500 for a non-key authentication on /v1/api-key; expired keys counting toward the limit; jOOQ self-reference clash. Evidence: docs/evidence/2026-10-24-api-keys.md</t>
+    <t xml:space="preserve">DoD: a revoked key is rejected on the very next request by identity (API test and browser e2e with a real Keycloak tenant admin, CI run 40084140187); other services may cache a verification for at most 30 s (Cache-Control: max-age=30; refusals no-store), so every service rejects it within 30 s. On EKS (run 40085243536): 87/87 checks, 107 resources applied and destroyed; /v1/api-key refuses no credentials, unknown keys and access tokens with no-store; V6 on RDS under forced RLS. Built: ADR-0010; keys mb_live_/mb_test_ + 238 random bits + CRC-32, SHA-256 at rest, shown once, never in idempotency records; one environment per key; scopes from a fixed vocabulary; expiry; rotation with a grace period; immediate revocation; 50 live keys per environment; last_used_at; keys cannot call the admin API. 193 tests (97.5% line / 87.1% branch). Found and fixed: timestamps serialised in the JVM zone instead of UTC; 500 for a non-key authentication on /v1/api-key; expired keys counting toward the limit; jOOQ self-reference clash. Evidence: docs/evidence/2026-10-24-api-keys.md | 2026-10-25: a real tenant admin signs in on EKS (PKCE) and a revoked key is rejected there.</t>
   </si>
   <si>
     <t xml:space="preserve">MB-T10</t>
@@ -819,7 +819,7 @@
     <t xml:space="preserve">https://github.com/mhrj7/meterbook/actions/runs/40091917398</t>
   </si>
   <si>
-    <t xml:space="preserve">DoD: plaintext pod-to-pod traffic is rejected. A pod outside the mesh, in the same namespace (admitted by the NetworkPolicy), is refused by strict mTLS; ztunnel logs 'explicitly denied by: istio-system/istio_converted_static_strict', asserted in the GitOps e2e on kind (CI run 40089193779, 34/34) and on EKS (run 40091917398: 107/107, 107 resources applied and destroyed). Control experiment: PERMISSIVE let the same plaintext pod through, STRICT refused it. In-mesh traffic carries SPIFFE identities, incl. identity -&gt; Keycloak as spiffe://cluster.local/ns/meterbook-dev/sa/identity. Built: ADR-0011 (Linkerd vs Istio sidecars vs Istio ambient); Istio 1.31.3 ambient via ArgoCD (charts from ghcr.io OCI, images from mirror.gcr.io); platform-mesh chart (STRICT, namespace enrolment from Git, never pruned); NetworkPolicies admit HBONE 15008 and mesh probe address only; render tests. Found and fixed: Istio 1.31 left gcr.io; ambient needs 15008 and 169.254.7.127 in NetworkPolicies; in-cluster verification lost output (kubectl run -i race), now run to completion and read from logs. Prod gets the mesh with its environment. Evidence: docs/evidence/2026-10-24-service-mesh-mtls.md</t>
+    <t xml:space="preserve">DoD: plaintext pod-to-pod traffic is rejected. A pod outside the mesh, in the same namespace (admitted by the NetworkPolicy), is refused by strict mTLS; ztunnel logs 'explicitly denied by: istio-system/istio_converted_static_strict', asserted in the GitOps e2e on kind (CI run 40089193779, 34/34) and on EKS (run 40091917398: 107/107, 107 resources applied and destroyed). Control experiment: PERMISSIVE let the same plaintext pod through, STRICT refused it. In-mesh traffic carries SPIFFE identities, incl. identity -&gt; Keycloak as spiffe://cluster.local/ns/meterbook-dev/sa/identity. Built: ADR-0011 (Linkerd vs Istio sidecars vs Istio ambient); Istio 1.31.3 ambient via ArgoCD (charts from ghcr.io OCI, images from mirror.gcr.io); platform-mesh chart (STRICT, namespace enrolment from Git, never pruned); NetworkPolicies admit HBONE 15008 and mesh probe address only; render tests. Found and fixed: Istio 1.31 left gcr.io; ambient needs 15008 and 169.254.7.127 in NetworkPolicies; in-cluster verification lost output (kubectl run -i race), now run to completion and read from logs. Prod gets the mesh with its environment. Evidence: docs/evidence/2026-10-24-service-mesh-mtls.md | 2026-10-25: TC-PLT-020 added; mTLS identities proven from ztunnel metrics; prod gets the mesh.</t>
   </si>
   <si>
     <t xml:space="preserve">MB-T11</t>
@@ -2043,6 +2043,12 @@
     <t xml:space="preserve">0 high/critical findings</t>
   </si>
   <si>
+    <t xml:space="preserve">CodeQL (security-extended; Java, Python, Actions) on every PR, main and weekly: 0 high/critical (a finding &gt;= 7.0 fails the run); Semgrep p/default on every change: 0 errors/warnings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/mhrj7/meterbook/actions/runs/40122321805</t>
+  </si>
+  <si>
     <t xml:space="preserve">TC-PLT-006</t>
   </si>
   <si>
@@ -2052,7 +2058,10 @@
     <t xml:space="preserve">Trivy</t>
   </si>
   <si>
-    <t xml:space="preserve">0 fixable CRITICAL in meterbook-identity; 1 unfixed CRITICAL in the distroless base (libbrotli1 CVE-2026-111497), tracked</t>
+    <t xml:space="preserve">0 CRITICAL, including unfixed, in all 4 deployed images (identity, Keycloak, db-bootstrap, smoke; Trivy 0.76.1, OS packages, jars, Go binaries); CI fails on fixable CRITICAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/mhrj7/meterbook/actions/runs/40115148732</t>
   </si>
   <si>
     <t xml:space="preserve">TC-PLT-007</t>
@@ -2142,6 +2151,12 @@
     <t xml:space="preserve">Linters in CI</t>
   </si>
   <si>
+    <t xml:space="preserve">This repo has Java, Python and shell (no Go or Rust): SpotBugs in ./gradlew check (found and fixed 5 real bugs; any finding fails), ruff and ShellCheck on every change; ci requires the job</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/mhrj7/meterbook/actions/runs/40122321801</t>
+  </si>
+  <si>
     <t xml:space="preserve">TC-PLT-014</t>
   </si>
   <si>
@@ -2523,6 +2538,42 @@
     <t xml:space="preserve">Custom generator</t>
   </si>
   <si>
+    <t xml:space="preserve">TC-PLT-020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service mesh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plaintext request from a pod outside the mesh to a meshed service in the same namespace (NetworkPolicy admits it)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refused by strict mTLS (ztunnel names the strict policy); in-mesh calls carry SPIFFE identities</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kind e2e + EKS verify</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refused with "explicitly denied by istio-system/istio_converted_static_strict"; PERMISSIVE control let the same pod through; identity -&gt; Keycloak counted as mutual_tls from spiffe://cluster.local/ns/meterbook-dev/sa/identity (EKS 123/123)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/mhrj7/meterbook/actions/runs/40117597732</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-PLT-021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Admission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deploy an image not signed by container.yml on main into an application namespace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refused at admission; every pinned image admitted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unsigned busybox refused ("no matching policies") in meterbook-*, allowed outside; all 4 pinned images pass a server-side dry run through the policy (EKS 123/123)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Metric ID</t>
   </si>
   <si>
@@ -2649,6 +2700,15 @@
     <t xml:space="preserve">count</t>
   </si>
   <si>
+    <t xml:space="preserve">Trivy 0.76.1 on the 4 pinned images</t>
+  </si>
+  <si>
+    <t xml:space="preserve">docs/evidence/2026-10-25-baseline-gaps.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRITICAL including unfixed; CI blocks fixable CRITICAL</t>
+  </si>
+  <si>
     <t xml:space="preserve">M-PLT-08</t>
   </si>
   <si>
@@ -3094,6 +3154,9 @@
   </si>
   <si>
     <t xml:space="preserve">identity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/mhrj7/meterbook/actions/runs/40120018649</t>
   </si>
   <si>
     <t xml:space="preserve">tenancy</t>
@@ -4281,54 +4344,54 @@
         <v>140</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>981</v>
+        <v>1002</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>982</v>
+        <v>1003</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>983</v>
+        <v>1004</v>
       </c>
       <c r="F1" s="13" t="s">
         <v>148</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>984</v>
+        <v>1005</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>985</v>
+        <v>1006</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>986</v>
+        <v>1007</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>987</v>
+        <v>1008</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>988</v>
+        <v>1009</v>
       </c>
       <c r="L1" s="13" t="s">
-        <v>989</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="s">
-        <v>990</v>
+        <v>1011</v>
       </c>
       <c r="B2" s="28" t="s">
         <v>157</v>
       </c>
       <c r="C2" s="28" t="s">
-        <v>991</v>
+        <v>1012</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>992</v>
+        <v>1013</v>
       </c>
       <c r="E2" s="28" t="s">
-        <v>700</v>
+        <v>705</v>
       </c>
       <c r="F2" s="28" t="s">
-        <v>985</v>
+        <v>1006</v>
       </c>
       <c r="G2" s="29" t="n">
         <v>46336</v>
@@ -4341,10 +4404,10 @@
         <v>1</v>
       </c>
       <c r="J2" s="28" t="s">
-        <v>993</v>
+        <v>1014</v>
       </c>
       <c r="K2" s="28" t="s">
-        <v>994</v>
+        <v>1015</v>
       </c>
       <c r="L2" s="28" t="s">
         <v>599</v>
@@ -6101,31 +6164,31 @@
         <v>145</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>995</v>
+        <v>1016</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>996</v>
+        <v>1017</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>997</v>
+        <v>1018</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>998</v>
+        <v>1019</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>999</v>
+        <v>1020</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>1000</v>
+        <v>1021</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>1001</v>
+        <v>1022</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>1002</v>
+        <v>1023</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>1003</v>
+        <v>1024</v>
       </c>
       <c r="K1" s="13" t="s">
         <v>594</v>
@@ -6755,7 +6818,7 @@
       </c>
       <c r="B17" s="18" t="n">
         <f aca="false">COUNTIF(Test_Cases!$B$2:$B$600,B$4)</f>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C17" s="18" t="n">
         <f aca="false">COUNTIF(Test_Cases!$B$2:$B$600,C$4)</f>
@@ -6763,7 +6826,7 @@
       </c>
       <c r="D17" s="19" t="n">
         <f aca="false">SUM(B17:C17)</f>
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6772,7 +6835,7 @@
       </c>
       <c r="B18" s="18" t="n">
         <f aca="false">COUNTIFS(Test_Cases!$B$2:$B$600,B$4,Test_Cases!$K$2:$K$600,"Pass")</f>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C18" s="18" t="n">
         <f aca="false">COUNTIFS(Test_Cases!$B$2:$B$600,C$4,Test_Cases!$K$2:$K$600,"Pass")</f>
@@ -6780,7 +6843,7 @@
       </c>
       <c r="D18" s="19" t="n">
         <f aca="false">SUM(B18:C18)</f>
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6823,7 +6886,7 @@
       </c>
       <c r="B21" s="18" t="n">
         <f aca="false">COUNTIFS(Test_Cases!$B$2:$B$600,B$4,Test_Cases!$K$2:$K$600,"Not Run")</f>
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C21" s="18" t="n">
         <f aca="false">COUNTIFS(Test_Cases!$B$2:$B$600,C$4,Test_Cases!$K$2:$K$600,"Not Run")</f>
@@ -6831,7 +6894,7 @@
       </c>
       <c r="D21" s="19" t="n">
         <f aca="false">SUM(B21:C21)</f>
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6840,7 +6903,7 @@
       </c>
       <c r="B22" s="22" t="n">
         <f aca="false">IFERROR((B17-B21)/B17,0)</f>
-        <v>0.315789473684211</v>
+        <v>0.476190476190476</v>
       </c>
       <c r="C22" s="22" t="n">
         <f aca="false">IFERROR((C17-C21)/C17,0)</f>
@@ -6848,7 +6911,7 @@
       </c>
       <c r="D22" s="22" t="n">
         <f aca="false">IFERROR((D17-D21)/D17,0)</f>
-        <v>0.133333333333333</v>
+        <v>0.212765957446809</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6916,7 +6979,7 @@
       </c>
       <c r="B28" s="18" t="n">
         <f aca="false">COUNTIFS(Metrics_SLOs!$B$2:$B$600,B$4,Metrics_SLOs!$I$2:$I$600,"PASS")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28" s="18" t="n">
         <f aca="false">COUNTIFS(Metrics_SLOs!$B$2:$B$600,C$4,Metrics_SLOs!$I$2:$I$600,"PASS")</f>
@@ -6924,7 +6987,7 @@
       </c>
       <c r="D28" s="19" t="n">
         <f aca="false">SUM(B28:C28)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6950,7 +7013,7 @@
       </c>
       <c r="B30" s="18" t="n">
         <f aca="false">COUNTIFS(Metrics_SLOs!$B$2:$B$600,B$4,Metrics_SLOs!$I$2:$I$600,"PENDING")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C30" s="18" t="n">
         <f aca="false">COUNTIFS(Metrics_SLOs!$B$2:$B$600,C$4,Metrics_SLOs!$I$2:$I$600,"PENDING")</f>
@@ -6958,7 +7021,7 @@
       </c>
       <c r="D30" s="19" t="n">
         <f aca="false">SUM(B30:C30)</f>
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7035,7 +7098,7 @@
       </c>
       <c r="B35" s="23" t="str">
         <f aca="false">COUNTIFS(Coverage!$A$2:$A$600,B$4,Coverage!$K$2:$K$600,"PASS")&amp;" / "&amp;COUNTIF(Coverage!$A$2:$A$600,B$4)</f>
-        <v>0 / 2</v>
+        <v>2 / 2</v>
       </c>
       <c r="C35" s="23" t="str">
         <f aca="false">COUNTIFS(Coverage!$A$2:$A$600,C$4,Coverage!$K$2:$K$600,"PASS")&amp;" / "&amp;COUNTIF(Coverage!$A$2:$A$600,C$4)</f>
@@ -7043,7 +7106,7 @@
       </c>
       <c r="D35" s="23" t="str">
         <f aca="false">(COUNTIF(Coverage!$K$2:$K$600,"PASS")-COUNTIFS(Coverage!$A$2:$A$600,"EXAMPLE",Coverage!$K$2:$K$600,"PASS"))&amp;" / "&amp;(COUNTA(Coverage!$A$2:$A$600)-COUNTIF(Coverage!$A$2:$A$600,"EXAMPLE"))</f>
-        <v>0 / 6</v>
+        <v>2 / 6</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7502,7 +7565,7 @@
       </c>
       <c r="D60" s="27" t="n">
         <f aca="false">COUNTIFS(Test_Cases!$C$2:$C$600,A60,Test_Cases!$K$2:$K$600,"Pass")-COUNTIFS(Test_Cases!$C$2:$C$600,A60,Test_Cases!$K$2:$K$600,"Pass",Test_Cases!$B$2:$B$600,"EXAMPLE")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E60" s="27" t="n">
         <f aca="false">COUNTIFS(Test_Cases!$C$2:$C$600,A60,Test_Cases!$K$2:$K$600,"Fail")-COUNTIFS(Test_Cases!$C$2:$C$600,A60,Test_Cases!$K$2:$K$600,"Fail",Test_Cases!$B$2:$B$600,"EXAMPLE")</f>
@@ -7510,7 +7573,7 @@
       </c>
       <c r="F60" s="27" t="n">
         <f aca="false">COUNTIFS(Test_Cases!$C$2:$C$600,A60,Test_Cases!$K$2:$K$600,"Not Run")-COUNTIFS(Test_Cases!$C$2:$C$600,A60,Test_Cases!$K$2:$K$600,"Not Run",Test_Cases!$B$2:$B$600,"EXAMPLE")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8052,7 +8115,7 @@
       </c>
       <c r="D82" s="27" t="n">
         <f aca="false">COUNTIFS(Test_Cases!$C$2:$C$600,A82,Test_Cases!$K$2:$K$600,"Pass")-COUNTIFS(Test_Cases!$C$2:$C$600,A82,Test_Cases!$K$2:$K$600,"Pass",Test_Cases!$B$2:$B$600,"EXAMPLE")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E82" s="27" t="n">
         <f aca="false">COUNTIFS(Test_Cases!$C$2:$C$600,A82,Test_Cases!$K$2:$K$600,"Fail")-COUNTIFS(Test_Cases!$C$2:$C$600,A82,Test_Cases!$K$2:$K$600,"Fail",Test_Cases!$B$2:$B$600,"EXAMPLE")</f>
@@ -8060,7 +8123,7 @@
       </c>
       <c r="F82" s="27" t="n">
         <f aca="false">COUNTIFS(Test_Cases!$C$2:$C$600,A82,Test_Cases!$K$2:$K$600,"Not Run")-COUNTIFS(Test_Cases!$C$2:$C$600,A82,Test_Cases!$K$2:$K$600,"Not Run",Test_Cases!$B$2:$B$600,"EXAMPLE")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8073,11 +8136,11 @@
       </c>
       <c r="C83" s="27" t="n">
         <f aca="false">COUNTIF(Test_Cases!$C$2:$C$600,A83)-COUNTIFS(Test_Cases!$C$2:$C$600,A83,Test_Cases!$B$2:$B$600,"EXAMPLE")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D83" s="27" t="n">
         <f aca="false">COUNTIFS(Test_Cases!$C$2:$C$600,A83,Test_Cases!$K$2:$K$600,"Pass")-COUNTIFS(Test_Cases!$C$2:$C$600,A83,Test_Cases!$K$2:$K$600,"Pass",Test_Cases!$B$2:$B$600,"EXAMPLE")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E83" s="27" t="n">
         <f aca="false">COUNTIFS(Test_Cases!$C$2:$C$600,A83,Test_Cases!$K$2:$K$600,"Fail")-COUNTIFS(Test_Cases!$C$2:$C$600,A83,Test_Cases!$K$2:$K$600,"Fail",Test_Cases!$B$2:$B$600,"EXAMPLE")</f>
@@ -8148,11 +8211,11 @@
       </c>
       <c r="C86" s="27" t="n">
         <f aca="false">COUNTIF(Test_Cases!$C$2:$C$600,A86)-COUNTIFS(Test_Cases!$C$2:$C$600,A86,Test_Cases!$B$2:$B$600,"EXAMPLE")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D86" s="27" t="n">
         <f aca="false">COUNTIFS(Test_Cases!$C$2:$C$600,A86,Test_Cases!$K$2:$K$600,"Pass")-COUNTIFS(Test_Cases!$C$2:$C$600,A86,Test_Cases!$K$2:$K$600,"Pass",Test_Cases!$B$2:$B$600,"EXAMPLE")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E86" s="27" t="n">
         <f aca="false">COUNTIFS(Test_Cases!$C$2:$C$600,A86,Test_Cases!$K$2:$K$600,"Fail")-COUNTIFS(Test_Cases!$C$2:$C$600,A86,Test_Cases!$K$2:$K$600,"Fail",Test_Cases!$B$2:$B$600,"EXAMPLE")</f>
@@ -8339,7 +8402,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{71B98949-D6D7-44F3-8360-3118E843C836}</x14:id>
+          <x14:id>{335289DB-DB61-408A-87EF-B07A376756B3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8353,7 +8416,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8219F0EC-4BDA-43B7-A77C-E3E6C200ADEE}</x14:id>
+          <x14:id>{C979CEB7-F435-4329-AD6E-5EECE5235CCE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8367,7 +8430,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D6F31996-A280-40E7-B386-25F134B1DBE6}</x14:id>
+          <x14:id>{14D6A86A-A5CA-43DB-BABA-C785A5B749CE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8381,7 +8444,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{607D3F38-9D15-4585-835C-6AD750874E71}</x14:id>
+          <x14:id>{86D04ABD-1823-45B5-A3D3-DA6F2BA3C52F}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8427,7 +8490,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{71B98949-D6D7-44F3-8360-3118E843C836}">
+          <x14:cfRule type="dataBar" id="{335289DB-DB61-408A-87EF-B07A376756B3}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -8442,7 +8505,7 @@
           <xm:sqref>B14:D14</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8219F0EC-4BDA-43B7-A77C-E3E6C200ADEE}">
+          <x14:cfRule type="dataBar" id="{C979CEB7-F435-4329-AD6E-5EECE5235CCE}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -8457,7 +8520,7 @@
           <xm:sqref>B22:D22</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D6F31996-A280-40E7-B386-25F134B1DBE6}">
+          <x14:cfRule type="dataBar" id="{14D6A86A-A5CA-43DB-BABA-C785A5B749CE}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -8472,7 +8535,7 @@
           <xm:sqref>B23:D23</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{607D3F38-9D15-4585-835C-6AD750874E71}">
+          <x14:cfRule type="dataBar" id="{86D04ABD-1823-45B5-A3D3-DA6F2BA3C52F}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -10655,7 +10718,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{F69AD8A5-E010-4990-B3A8-E2E633EE8FBA}</x14:id>
+          <x14:id>{A4B27AF6-B282-44F5-988D-F9DA739DB031}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10686,7 +10749,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{F69AD8A5-E010-4990-B3A8-E2E633EE8FBA}">
+          <x14:cfRule type="dataBar" id="{A4B27AF6-B282-44F5-988D-F9DA739DB031}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -12438,7 +12501,7 @@
     <tabColor rgb="FF548235"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O47"/>
+  <dimension ref="A1:O49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
@@ -12762,16 +12825,22 @@
         <v>599</v>
       </c>
       <c r="K7" s="33" t="s">
-        <v>68</v>
-      </c>
-      <c r="L7" s="36"/>
-      <c r="M7" s="33"/>
+        <v>378</v>
+      </c>
+      <c r="L7" s="36" t="n">
+        <v>46320</v>
+      </c>
+      <c r="M7" s="33" t="s">
+        <v>626</v>
+      </c>
       <c r="N7" s="33"/>
-      <c r="O7" s="33"/>
+      <c r="O7" s="33" t="s">
+        <v>627</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="31" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="B8" s="31" t="s">
         <v>5</v>
@@ -12787,13 +12856,13 @@
         <v>623</v>
       </c>
       <c r="F8" s="31" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="G8" s="31" t="s">
         <v>543</v>
       </c>
       <c r="H8" s="31" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="I8" s="31" t="s">
         <v>161</v>
@@ -12805,19 +12874,19 @@
         <v>378</v>
       </c>
       <c r="L8" s="36" t="n">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="M8" s="33" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="N8" s="33"/>
       <c r="O8" s="33" t="s">
-        <v>189</v>
+        <v>632</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="31" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="B9" s="31" t="s">
         <v>5</v>
@@ -12833,7 +12902,7 @@
         <v>623</v>
       </c>
       <c r="F9" s="31" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="G9" s="31" t="s">
         <v>547</v>
@@ -12854,16 +12923,16 @@
         <v>46318</v>
       </c>
       <c r="M9" s="33" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
       <c r="N9" s="33"/>
       <c r="O9" s="33" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="31" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="B10" s="31" t="s">
         <v>5</v>
@@ -12876,10 +12945,10 @@
         <v>Black</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="F10" s="31" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="G10" s="31" t="s">
         <v>551</v>
@@ -12903,7 +12972,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="31" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
       <c r="B11" s="31" t="s">
         <v>5</v>
@@ -12916,13 +12985,13 @@
         <v>Black</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="F11" s="31" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="G11" s="31" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
       <c r="H11" s="31" t="s">
         <v>372</v>
@@ -12943,7 +13012,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="31" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
       <c r="B12" s="31" t="s">
         <v>5</v>
@@ -12956,16 +13025,16 @@
         <v>Grey</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="F12" s="31" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="G12" s="31" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
       <c r="H12" s="31" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="I12" s="31" t="s">
         <v>161</v>
@@ -12983,7 +13052,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="31" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="B13" s="31" t="s">
         <v>5</v>
@@ -12996,13 +13065,13 @@
         <v>Grey</v>
       </c>
       <c r="E13" s="31" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="G13" s="31" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="H13" s="31" t="s">
         <v>554</v>
@@ -13023,7 +13092,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="31" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="B14" s="31" t="s">
         <v>5</v>
@@ -13036,16 +13105,16 @@
         <v>Grey</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
       <c r="F14" s="31" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="G14" s="31" t="s">
-        <v>653</v>
+        <v>656</v>
       </c>
       <c r="H14" s="31" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="I14" s="31" t="s">
         <v>161</v>
@@ -13063,7 +13132,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="31" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="B15" s="31" t="s">
         <v>5</v>
@@ -13079,13 +13148,13 @@
         <v>623</v>
       </c>
       <c r="F15" s="31" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="G15" s="31" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
       <c r="H15" s="31" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="I15" s="31" t="s">
         <v>161</v>
@@ -13094,16 +13163,22 @@
         <v>599</v>
       </c>
       <c r="K15" s="33" t="s">
-        <v>68</v>
-      </c>
-      <c r="L15" s="36"/>
-      <c r="M15" s="33"/>
+        <v>378</v>
+      </c>
+      <c r="L15" s="36" t="n">
+        <v>46320</v>
+      </c>
+      <c r="M15" s="33" t="s">
+        <v>662</v>
+      </c>
       <c r="N15" s="33"/>
-      <c r="O15" s="33"/>
+      <c r="O15" s="33" t="s">
+        <v>663</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="31" t="s">
-        <v>659</v>
+        <v>664</v>
       </c>
       <c r="B16" s="31" t="s">
         <v>5</v>
@@ -13119,13 +13194,13 @@
         <v>623</v>
       </c>
       <c r="F16" s="31" t="s">
-        <v>660</v>
+        <v>665</v>
       </c>
       <c r="G16" s="31" t="s">
-        <v>661</v>
+        <v>666</v>
       </c>
       <c r="H16" s="31" t="s">
-        <v>662</v>
+        <v>667</v>
       </c>
       <c r="I16" s="31" t="s">
         <v>161</v>
@@ -13140,7 +13215,7 @@
         <v>46319</v>
       </c>
       <c r="M16" s="33" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="N16" s="33"/>
       <c r="O16" s="33" t="s">
@@ -13149,7 +13224,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="31" t="s">
-        <v>664</v>
+        <v>669</v>
       </c>
       <c r="B17" s="31" t="s">
         <v>5</v>
@@ -13162,16 +13237,16 @@
         <v>Black</v>
       </c>
       <c r="E17" s="31" t="s">
-        <v>665</v>
+        <v>670</v>
       </c>
       <c r="F17" s="31" t="s">
-        <v>666</v>
+        <v>671</v>
       </c>
       <c r="G17" s="31" t="s">
-        <v>667</v>
+        <v>672</v>
       </c>
       <c r="H17" s="31" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="I17" s="31" t="s">
         <v>168</v>
@@ -13189,7 +13264,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="31" t="s">
-        <v>669</v>
+        <v>674</v>
       </c>
       <c r="B18" s="31" t="s">
         <v>5</v>
@@ -13202,13 +13277,13 @@
         <v>Grey</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="F18" s="31" t="s">
-        <v>670</v>
+        <v>675</v>
       </c>
       <c r="G18" s="31" t="s">
-        <v>671</v>
+        <v>676</v>
       </c>
       <c r="H18" s="31" t="s">
         <v>509</v>
@@ -13229,7 +13304,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="31" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="B19" s="31" t="s">
         <v>5</v>
@@ -13242,16 +13317,16 @@
         <v>Grey</v>
       </c>
       <c r="E19" s="31" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="F19" s="31" t="s">
-        <v>674</v>
+        <v>679</v>
       </c>
       <c r="G19" s="31" t="s">
-        <v>675</v>
+        <v>680</v>
       </c>
       <c r="H19" s="31" t="s">
-        <v>676</v>
+        <v>681</v>
       </c>
       <c r="I19" s="31" t="s">
         <v>168</v>
@@ -13269,7 +13344,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="31" t="s">
-        <v>677</v>
+        <v>682</v>
       </c>
       <c r="B20" s="31" t="s">
         <v>5</v>
@@ -13285,13 +13360,13 @@
         <v>5</v>
       </c>
       <c r="F20" s="31" t="s">
-        <v>678</v>
+        <v>683</v>
       </c>
       <c r="G20" s="31" t="s">
-        <v>679</v>
+        <v>684</v>
       </c>
       <c r="H20" s="31" t="s">
-        <v>680</v>
+        <v>685</v>
       </c>
       <c r="I20" s="31" t="s">
         <v>238</v>
@@ -13309,7 +13384,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>681</v>
+        <v>686</v>
       </c>
       <c r="B21" s="31" t="s">
         <v>5</v>
@@ -13322,10 +13397,10 @@
         <v>Black</v>
       </c>
       <c r="E21" s="31" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="F21" s="31" t="s">
-        <v>682</v>
+        <v>687</v>
       </c>
       <c r="G21" s="31" t="s">
         <v>559</v>
@@ -13349,7 +13424,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="31" t="s">
-        <v>683</v>
+        <v>688</v>
       </c>
       <c r="B22" s="31" t="s">
         <v>7</v>
@@ -13362,16 +13437,16 @@
         <v>White</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>684</v>
+        <v>689</v>
       </c>
       <c r="F22" s="31" t="s">
-        <v>685</v>
+        <v>690</v>
       </c>
       <c r="G22" s="31" t="s">
-        <v>686</v>
+        <v>691</v>
       </c>
       <c r="H22" s="31" t="s">
-        <v>687</v>
+        <v>692</v>
       </c>
       <c r="I22" s="31" t="s">
         <v>161</v>
@@ -13389,7 +13464,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="31" t="s">
-        <v>688</v>
+        <v>693</v>
       </c>
       <c r="B23" s="31" t="s">
         <v>7</v>
@@ -13402,13 +13477,13 @@
         <v>White</v>
       </c>
       <c r="E23" s="31" t="s">
-        <v>689</v>
+        <v>694</v>
       </c>
       <c r="F23" s="31" t="s">
-        <v>690</v>
+        <v>695</v>
       </c>
       <c r="G23" s="31" t="s">
-        <v>691</v>
+        <v>696</v>
       </c>
       <c r="H23" s="31" t="s">
         <v>421</v>
@@ -13429,7 +13504,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="31" t="s">
-        <v>692</v>
+        <v>697</v>
       </c>
       <c r="B24" s="31" t="s">
         <v>7</v>
@@ -13442,16 +13517,16 @@
         <v>White</v>
       </c>
       <c r="E24" s="31" t="s">
-        <v>684</v>
+        <v>689</v>
       </c>
       <c r="F24" s="31" t="s">
-        <v>693</v>
+        <v>698</v>
       </c>
       <c r="G24" s="31" t="s">
-        <v>694</v>
+        <v>699</v>
       </c>
       <c r="H24" s="31" t="s">
-        <v>695</v>
+        <v>700</v>
       </c>
       <c r="I24" s="31" t="s">
         <v>168</v>
@@ -13469,7 +13544,7 @@
     </row>
     <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="31" t="s">
-        <v>696</v>
+        <v>701</v>
       </c>
       <c r="B25" s="31" t="s">
         <v>7</v>
@@ -13482,13 +13557,13 @@
         <v>Black</v>
       </c>
       <c r="E25" s="31" t="s">
-        <v>697</v>
+        <v>702</v>
       </c>
       <c r="F25" s="31" t="s">
-        <v>698</v>
+        <v>703</v>
       </c>
       <c r="G25" s="31" t="s">
-        <v>699</v>
+        <v>704</v>
       </c>
       <c r="H25" s="31" t="s">
         <v>351</v>
@@ -13509,7 +13584,7 @@
     </row>
     <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="31" t="s">
-        <v>700</v>
+        <v>705</v>
       </c>
       <c r="B26" s="31" t="s">
         <v>7</v>
@@ -13525,10 +13600,10 @@
         <v>596</v>
       </c>
       <c r="F26" s="31" t="s">
-        <v>701</v>
+        <v>706</v>
       </c>
       <c r="G26" s="31" t="s">
-        <v>702</v>
+        <v>707</v>
       </c>
       <c r="H26" s="31" t="s">
         <v>442</v>
@@ -13549,7 +13624,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="31" t="s">
-        <v>703</v>
+        <v>708</v>
       </c>
       <c r="B27" s="31" t="s">
         <v>7</v>
@@ -13562,16 +13637,16 @@
         <v>White</v>
       </c>
       <c r="E27" s="31" t="s">
-        <v>689</v>
+        <v>694</v>
       </c>
       <c r="F27" s="31" t="s">
-        <v>704</v>
+        <v>709</v>
       </c>
       <c r="G27" s="31" t="s">
-        <v>705</v>
+        <v>710</v>
       </c>
       <c r="H27" s="31" t="s">
-        <v>706</v>
+        <v>711</v>
       </c>
       <c r="I27" s="31" t="s">
         <v>161</v>
@@ -13589,7 +13664,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="31" t="s">
-        <v>707</v>
+        <v>712</v>
       </c>
       <c r="B28" s="31" t="s">
         <v>7</v>
@@ -13602,13 +13677,13 @@
         <v>Black</v>
       </c>
       <c r="E28" s="31" t="s">
-        <v>708</v>
+        <v>713</v>
       </c>
       <c r="F28" s="31" t="s">
-        <v>709</v>
+        <v>714</v>
       </c>
       <c r="G28" s="31" t="s">
-        <v>710</v>
+        <v>715</v>
       </c>
       <c r="H28" s="31" t="s">
         <v>344</v>
@@ -13629,7 +13704,7 @@
     </row>
     <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="31" t="s">
-        <v>711</v>
+        <v>716</v>
       </c>
       <c r="B29" s="31" t="s">
         <v>7</v>
@@ -13642,16 +13717,16 @@
         <v>Grey</v>
       </c>
       <c r="E29" s="31" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="F29" s="31" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="G29" s="31" t="s">
-        <v>714</v>
+        <v>719</v>
       </c>
       <c r="H29" s="31" t="s">
-        <v>715</v>
+        <v>720</v>
       </c>
       <c r="I29" s="31" t="s">
         <v>161</v>
@@ -13669,7 +13744,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="31" t="s">
-        <v>716</v>
+        <v>721</v>
       </c>
       <c r="B30" s="31" t="s">
         <v>7</v>
@@ -13682,16 +13757,16 @@
         <v>Black</v>
       </c>
       <c r="E30" s="31" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
       <c r="F30" s="31" t="s">
-        <v>718</v>
+        <v>723</v>
       </c>
       <c r="G30" s="31" t="s">
-        <v>719</v>
+        <v>724</v>
       </c>
       <c r="H30" s="31" t="s">
-        <v>720</v>
+        <v>725</v>
       </c>
       <c r="I30" s="31" t="s">
         <v>161</v>
@@ -13709,7 +13784,7 @@
     </row>
     <row r="31" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="31" t="s">
-        <v>721</v>
+        <v>726</v>
       </c>
       <c r="B31" s="31" t="s">
         <v>7</v>
@@ -13722,13 +13797,13 @@
         <v>Black</v>
       </c>
       <c r="E31" s="31" t="s">
-        <v>722</v>
+        <v>727</v>
       </c>
       <c r="F31" s="31" t="s">
-        <v>723</v>
+        <v>728</v>
       </c>
       <c r="G31" s="31" t="s">
-        <v>724</v>
+        <v>729</v>
       </c>
       <c r="H31" s="31" t="s">
         <v>391</v>
@@ -13749,7 +13824,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="31" t="s">
-        <v>725</v>
+        <v>730</v>
       </c>
       <c r="B32" s="31" t="s">
         <v>7</v>
@@ -13762,13 +13837,13 @@
         <v>White</v>
       </c>
       <c r="E32" s="31" t="s">
-        <v>726</v>
+        <v>731</v>
       </c>
       <c r="F32" s="31" t="s">
-        <v>727</v>
+        <v>732</v>
       </c>
       <c r="G32" s="31" t="s">
-        <v>728</v>
+        <v>733</v>
       </c>
       <c r="H32" s="31" t="s">
         <v>429</v>
@@ -13789,7 +13864,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="31" t="s">
-        <v>729</v>
+        <v>734</v>
       </c>
       <c r="B33" s="31" t="s">
         <v>7</v>
@@ -13802,13 +13877,13 @@
         <v>Black</v>
       </c>
       <c r="E33" s="31" t="s">
-        <v>730</v>
+        <v>735</v>
       </c>
       <c r="F33" s="31" t="s">
-        <v>731</v>
+        <v>736</v>
       </c>
       <c r="G33" s="31" t="s">
-        <v>732</v>
+        <v>737</v>
       </c>
       <c r="H33" s="31" t="s">
         <v>366</v>
@@ -13829,7 +13904,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="31" t="s">
-        <v>733</v>
+        <v>738</v>
       </c>
       <c r="B34" s="31" t="s">
         <v>7</v>
@@ -13842,16 +13917,16 @@
         <v>Grey</v>
       </c>
       <c r="E34" s="31" t="s">
-        <v>734</v>
+        <v>739</v>
       </c>
       <c r="F34" s="31" t="s">
-        <v>735</v>
+        <v>740</v>
       </c>
       <c r="G34" s="31" t="s">
-        <v>736</v>
+        <v>741</v>
       </c>
       <c r="H34" s="31" t="s">
-        <v>737</v>
+        <v>742</v>
       </c>
       <c r="I34" s="31" t="s">
         <v>161</v>
@@ -13869,7 +13944,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="31" t="s">
-        <v>738</v>
+        <v>743</v>
       </c>
       <c r="B35" s="31" t="s">
         <v>7</v>
@@ -13882,13 +13957,13 @@
         <v>Black</v>
       </c>
       <c r="E35" s="31" t="s">
-        <v>708</v>
+        <v>713</v>
       </c>
       <c r="F35" s="31" t="s">
-        <v>739</v>
+        <v>744</v>
       </c>
       <c r="G35" s="31" t="s">
-        <v>740</v>
+        <v>745</v>
       </c>
       <c r="H35" s="31" t="s">
         <v>554</v>
@@ -13909,7 +13984,7 @@
     </row>
     <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="31" t="s">
-        <v>741</v>
+        <v>746</v>
       </c>
       <c r="B36" s="31" t="s">
         <v>7</v>
@@ -13922,13 +13997,13 @@
         <v>Grey</v>
       </c>
       <c r="E36" s="31" t="s">
-        <v>742</v>
+        <v>747</v>
       </c>
       <c r="F36" s="31" t="s">
-        <v>743</v>
+        <v>748</v>
       </c>
       <c r="G36" s="31" t="s">
-        <v>744</v>
+        <v>749</v>
       </c>
       <c r="H36" s="31" t="s">
         <v>451</v>
@@ -13949,7 +14024,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="31" t="s">
-        <v>745</v>
+        <v>750</v>
       </c>
       <c r="B37" s="31" t="s">
         <v>7</v>
@@ -13962,10 +14037,10 @@
         <v>Black</v>
       </c>
       <c r="E37" s="31" t="s">
-        <v>746</v>
+        <v>751</v>
       </c>
       <c r="F37" s="31" t="s">
-        <v>747</v>
+        <v>752</v>
       </c>
       <c r="G37" s="31" t="s">
         <v>388</v>
@@ -13989,7 +14064,7 @@
     </row>
     <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="31" t="s">
-        <v>748</v>
+        <v>753</v>
       </c>
       <c r="B38" s="31" t="s">
         <v>7</v>
@@ -14002,16 +14077,16 @@
         <v>Grey</v>
       </c>
       <c r="E38" s="31" t="s">
-        <v>749</v>
+        <v>754</v>
       </c>
       <c r="F38" s="31" t="s">
-        <v>750</v>
+        <v>755</v>
       </c>
       <c r="G38" s="31" t="s">
-        <v>751</v>
+        <v>756</v>
       </c>
       <c r="H38" s="31" t="s">
-        <v>752</v>
+        <v>757</v>
       </c>
       <c r="I38" s="31" t="s">
         <v>161</v>
@@ -14029,7 +14104,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="31" t="s">
-        <v>753</v>
+        <v>758</v>
       </c>
       <c r="B39" s="31" t="s">
         <v>7</v>
@@ -14042,13 +14117,13 @@
         <v>Black</v>
       </c>
       <c r="E39" s="31" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="F39" s="31" t="s">
-        <v>754</v>
+        <v>759</v>
       </c>
       <c r="G39" s="31" t="s">
-        <v>755</v>
+        <v>760</v>
       </c>
       <c r="H39" s="31" t="s">
         <v>353</v>
@@ -14069,7 +14144,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="31" t="s">
-        <v>756</v>
+        <v>761</v>
       </c>
       <c r="B40" s="31" t="s">
         <v>7</v>
@@ -14082,13 +14157,13 @@
         <v>Black</v>
       </c>
       <c r="E40" s="31" t="s">
-        <v>730</v>
+        <v>735</v>
       </c>
       <c r="F40" s="31" t="s">
-        <v>757</v>
+        <v>762</v>
       </c>
       <c r="G40" s="31" t="s">
-        <v>758</v>
+        <v>763</v>
       </c>
       <c r="H40" s="31" t="s">
         <v>572</v>
@@ -14109,7 +14184,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="31" t="s">
-        <v>759</v>
+        <v>764</v>
       </c>
       <c r="B41" s="31" t="s">
         <v>7</v>
@@ -14122,16 +14197,16 @@
         <v>Black</v>
       </c>
       <c r="E41" s="31" t="s">
-        <v>760</v>
+        <v>765</v>
       </c>
       <c r="F41" s="31" t="s">
-        <v>761</v>
+        <v>766</v>
       </c>
       <c r="G41" s="31" t="s">
-        <v>762</v>
+        <v>767</v>
       </c>
       <c r="H41" s="31" t="s">
-        <v>763</v>
+        <v>768</v>
       </c>
       <c r="I41" s="31" t="s">
         <v>168</v>
@@ -14149,7 +14224,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="31" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B42" s="31" t="s">
         <v>7</v>
@@ -14162,13 +14237,13 @@
         <v>Black</v>
       </c>
       <c r="E42" s="31" t="s">
-        <v>765</v>
+        <v>770</v>
       </c>
       <c r="F42" s="31" t="s">
-        <v>766</v>
+        <v>771</v>
       </c>
       <c r="G42" s="31" t="s">
-        <v>767</v>
+        <v>772</v>
       </c>
       <c r="H42" s="31" t="s">
         <v>470</v>
@@ -14189,7 +14264,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="31" t="s">
-        <v>768</v>
+        <v>773</v>
       </c>
       <c r="B43" s="31" t="s">
         <v>7</v>
@@ -14202,13 +14277,13 @@
         <v>Black</v>
       </c>
       <c r="E43" s="31" t="s">
-        <v>765</v>
+        <v>770</v>
       </c>
       <c r="F43" s="31" t="s">
-        <v>769</v>
+        <v>774</v>
       </c>
       <c r="G43" s="31" t="s">
-        <v>770</v>
+        <v>775</v>
       </c>
       <c r="H43" s="31" t="s">
         <v>470</v>
@@ -14229,7 +14304,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="31" t="s">
-        <v>771</v>
+        <v>776</v>
       </c>
       <c r="B44" s="31" t="s">
         <v>7</v>
@@ -14242,13 +14317,13 @@
         <v>Black</v>
       </c>
       <c r="E44" s="31" t="s">
-        <v>772</v>
+        <v>777</v>
       </c>
       <c r="F44" s="31" t="s">
-        <v>773</v>
+        <v>778</v>
       </c>
       <c r="G44" s="31" t="s">
-        <v>774</v>
+        <v>779</v>
       </c>
       <c r="H44" s="31" t="s">
         <v>470</v>
@@ -14269,7 +14344,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="31" t="s">
-        <v>775</v>
+        <v>780</v>
       </c>
       <c r="B45" s="31" t="s">
         <v>7</v>
@@ -14282,13 +14357,13 @@
         <v>Black</v>
       </c>
       <c r="E45" s="31" t="s">
-        <v>776</v>
+        <v>781</v>
       </c>
       <c r="F45" s="31" t="s">
-        <v>777</v>
+        <v>782</v>
       </c>
       <c r="G45" s="31" t="s">
-        <v>778</v>
+        <v>783</v>
       </c>
       <c r="H45" s="31" t="s">
         <v>483</v>
@@ -14309,7 +14384,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="31" t="s">
-        <v>779</v>
+        <v>784</v>
       </c>
       <c r="B46" s="31" t="s">
         <v>7</v>
@@ -14322,13 +14397,13 @@
         <v>Black</v>
       </c>
       <c r="E46" s="31" t="s">
-        <v>765</v>
+        <v>770</v>
       </c>
       <c r="F46" s="31" t="s">
-        <v>780</v>
+        <v>785</v>
       </c>
       <c r="G46" s="31" t="s">
-        <v>781</v>
+        <v>786</v>
       </c>
       <c r="H46" s="31" t="s">
         <v>470</v>
@@ -14349,7 +14424,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="31" t="s">
-        <v>782</v>
+        <v>787</v>
       </c>
       <c r="B47" s="31" t="s">
         <v>7</v>
@@ -14362,16 +14437,16 @@
         <v>Black</v>
       </c>
       <c r="E47" s="31" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
       <c r="F47" s="31" t="s">
-        <v>783</v>
+        <v>788</v>
       </c>
       <c r="G47" s="31" t="s">
-        <v>784</v>
+        <v>789</v>
       </c>
       <c r="H47" s="31" t="s">
-        <v>785</v>
+        <v>790</v>
       </c>
       <c r="I47" s="31" t="s">
         <v>168</v>
@@ -14386,6 +14461,98 @@
       <c r="M47" s="33"/>
       <c r="N47" s="33"/>
       <c r="O47" s="33"/>
+    </row>
+    <row r="48" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="31" t="s">
+        <v>791</v>
+      </c>
+      <c r="B48" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="C48" s="31" t="s">
+        <v>131</v>
+      </c>
+      <c r="D48" s="31" t="str">
+        <f aca="false">IFERROR(INDEX(Test_Catalog!$C$2:$C$48,MATCH(C48,Test_Catalog!$A$2:$A$48,0)),"")</f>
+        <v>Black</v>
+      </c>
+      <c r="E48" s="31" t="s">
+        <v>792</v>
+      </c>
+      <c r="F48" s="31" t="s">
+        <v>793</v>
+      </c>
+      <c r="G48" s="31" t="s">
+        <v>794</v>
+      </c>
+      <c r="H48" s="31" t="s">
+        <v>795</v>
+      </c>
+      <c r="I48" s="31" t="s">
+        <v>168</v>
+      </c>
+      <c r="J48" s="33" t="s">
+        <v>599</v>
+      </c>
+      <c r="K48" s="33" t="s">
+        <v>378</v>
+      </c>
+      <c r="L48" s="36" t="n">
+        <v>46320</v>
+      </c>
+      <c r="M48" s="33" t="s">
+        <v>796</v>
+      </c>
+      <c r="N48" s="33"/>
+      <c r="O48" s="33" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="31" t="s">
+        <v>798</v>
+      </c>
+      <c r="B49" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="C49" s="31" t="s">
+        <v>128</v>
+      </c>
+      <c r="D49" s="31" t="str">
+        <f aca="false">IFERROR(INDEX(Test_Catalog!$C$2:$C$48,MATCH(C49,Test_Catalog!$A$2:$A$48,0)),"")</f>
+        <v>White</v>
+      </c>
+      <c r="E49" s="31" t="s">
+        <v>799</v>
+      </c>
+      <c r="F49" s="31" t="s">
+        <v>800</v>
+      </c>
+      <c r="G49" s="31" t="s">
+        <v>801</v>
+      </c>
+      <c r="H49" s="31" t="s">
+        <v>795</v>
+      </c>
+      <c r="I49" s="31" t="s">
+        <v>161</v>
+      </c>
+      <c r="J49" s="33" t="s">
+        <v>599</v>
+      </c>
+      <c r="K49" s="33" t="s">
+        <v>378</v>
+      </c>
+      <c r="L49" s="36" t="n">
+        <v>46320</v>
+      </c>
+      <c r="M49" s="33" t="s">
+        <v>802</v>
+      </c>
+      <c r="N49" s="33"/>
+      <c r="O49" s="33" t="s">
+        <v>797</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O600"/>
@@ -14454,7 +14621,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>786</v>
+        <v>803</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>140</v>
@@ -14463,31 +14630,31 @@
         <v>310</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>787</v>
+        <v>804</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>788</v>
+        <v>805</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>789</v>
+        <v>806</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>91</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>790</v>
+        <v>807</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>791</v>
+        <v>808</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>792</v>
+        <v>809</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>793</v>
+        <v>810</v>
       </c>
       <c r="L1" s="13" t="s">
-        <v>794</v>
+        <v>811</v>
       </c>
       <c r="M1" s="13" t="s">
         <v>594</v>
@@ -14498,7 +14665,7 @@
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="s">
-        <v>795</v>
+        <v>812</v>
       </c>
       <c r="B2" s="28" t="s">
         <v>157</v>
@@ -14507,16 +14674,16 @@
         <v>42</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>796</v>
+        <v>813</v>
       </c>
       <c r="E2" s="28" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="F2" s="37" t="n">
         <v>50</v>
       </c>
       <c r="G2" s="28" t="s">
-        <v>798</v>
+        <v>815</v>
       </c>
       <c r="H2" s="37" t="n">
         <v>38</v>
@@ -14529,37 +14696,37 @@
         <v>470</v>
       </c>
       <c r="K2" s="28" t="s">
-        <v>799</v>
+        <v>816</v>
       </c>
       <c r="L2" s="29" t="n">
         <v>46338</v>
       </c>
       <c r="M2" s="28" t="s">
-        <v>800</v>
+        <v>817</v>
       </c>
       <c r="N2" s="28"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="31" t="s">
-        <v>801</v>
+        <v>818</v>
       </c>
       <c r="B3" s="31" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>802</v>
+        <v>819</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>803</v>
+        <v>820</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>804</v>
+        <v>821</v>
       </c>
       <c r="F3" s="38" t="n">
         <v>0.999</v>
       </c>
       <c r="G3" s="31" t="s">
-        <v>805</v>
+        <v>822</v>
       </c>
       <c r="H3" s="39"/>
       <c r="I3" s="31" t="str">
@@ -14567,7 +14734,7 @@
         <v>PENDING</v>
       </c>
       <c r="J3" s="31" t="s">
-        <v>806</v>
+        <v>823</v>
       </c>
       <c r="K3" s="33"/>
       <c r="L3" s="36"/>
@@ -14576,7 +14743,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>807</v>
+        <v>824</v>
       </c>
       <c r="B4" s="31" t="s">
         <v>5</v>
@@ -14585,16 +14752,16 @@
         <v>42</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>808</v>
+        <v>825</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="F4" s="40" t="n">
         <v>300</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>798</v>
+        <v>815</v>
       </c>
       <c r="H4" s="41"/>
       <c r="I4" s="31" t="str">
@@ -14611,25 +14778,25 @@
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>809</v>
+        <v>826</v>
       </c>
       <c r="B5" s="31" t="s">
         <v>5</v>
       </c>
       <c r="C5" s="31" t="s">
-        <v>810</v>
+        <v>827</v>
       </c>
       <c r="D5" s="31" t="s">
-        <v>811</v>
+        <v>828</v>
       </c>
       <c r="E5" s="31" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="F5" s="40" t="n">
         <v>10</v>
       </c>
       <c r="G5" s="31" t="s">
-        <v>812</v>
+        <v>829</v>
       </c>
       <c r="H5" s="41" t="n">
         <v>3.3</v>
@@ -14639,42 +14806,42 @@
         <v>PASS</v>
       </c>
       <c r="J5" s="31" t="s">
-        <v>813</v>
+        <v>830</v>
       </c>
       <c r="K5" s="33" t="s">
-        <v>814</v>
+        <v>831</v>
       </c>
       <c r="L5" s="36" t="n">
         <v>46318</v>
       </c>
       <c r="M5" s="33" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="N5" s="33" t="s">
-        <v>815</v>
+        <v>832</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="31" t="s">
-        <v>816</v>
+        <v>833</v>
       </c>
       <c r="B6" s="31" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>810</v>
+        <v>827</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>817</v>
+        <v>834</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>804</v>
+        <v>821</v>
       </c>
       <c r="F6" s="40" t="n">
         <v>5</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>818</v>
+        <v>835</v>
       </c>
       <c r="H6" s="41"/>
       <c r="I6" s="31" t="str">
@@ -14682,7 +14849,7 @@
         <v>PENDING</v>
       </c>
       <c r="J6" s="31" t="s">
-        <v>819</v>
+        <v>836</v>
       </c>
       <c r="K6" s="33"/>
       <c r="L6" s="36"/>
@@ -14691,25 +14858,25 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="31" t="s">
-        <v>820</v>
+        <v>837</v>
       </c>
       <c r="B7" s="31" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="31" t="s">
-        <v>810</v>
+        <v>827</v>
       </c>
       <c r="D7" s="31" t="s">
-        <v>821</v>
+        <v>838</v>
       </c>
       <c r="E7" s="31" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="F7" s="38" t="n">
         <v>0.15</v>
       </c>
       <c r="G7" s="31" t="s">
-        <v>805</v>
+        <v>822</v>
       </c>
       <c r="H7" s="39"/>
       <c r="I7" s="31" t="str">
@@ -14717,7 +14884,7 @@
         <v>PENDING</v>
       </c>
       <c r="J7" s="31" t="s">
-        <v>822</v>
+        <v>839</v>
       </c>
       <c r="K7" s="33"/>
       <c r="L7" s="36"/>
@@ -14726,25 +14893,25 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="31" t="s">
-        <v>823</v>
+        <v>840</v>
       </c>
       <c r="B8" s="31" t="s">
         <v>5</v>
       </c>
       <c r="C8" s="31" t="s">
-        <v>810</v>
+        <v>827</v>
       </c>
       <c r="D8" s="31" t="s">
-        <v>824</v>
+        <v>841</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="F8" s="40" t="n">
         <v>30</v>
       </c>
       <c r="G8" s="31" t="s">
-        <v>812</v>
+        <v>829</v>
       </c>
       <c r="H8" s="41"/>
       <c r="I8" s="31" t="str">
@@ -14752,7 +14919,7 @@
         <v>PENDING</v>
       </c>
       <c r="J8" s="31" t="s">
-        <v>822</v>
+        <v>839</v>
       </c>
       <c r="K8" s="33"/>
       <c r="L8" s="36"/>
@@ -14761,7 +14928,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="31" t="s">
-        <v>825</v>
+        <v>842</v>
       </c>
       <c r="B9" s="31" t="s">
         <v>5</v>
@@ -14770,51 +14937,61 @@
         <v>209</v>
       </c>
       <c r="D9" s="31" t="s">
-        <v>826</v>
+        <v>843</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="F9" s="40" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="31" t="s">
-        <v>827</v>
-      </c>
-      <c r="H9" s="41"/>
+        <v>844</v>
+      </c>
+      <c r="H9" s="41" t="n">
+        <v>0</v>
+      </c>
       <c r="I9" s="31" t="str">
         <f aca="false">IF(H9="","PENDING",IF(E9="&lt;=",IF(H9&lt;=F9,"PASS","FAIL"),IF(H9&gt;=F9,"PASS","FAIL")))</f>
-        <v>PENDING</v>
+        <v>PASS</v>
       </c>
       <c r="J9" s="31" t="s">
-        <v>628</v>
-      </c>
-      <c r="K9" s="33"/>
-      <c r="L9" s="36"/>
-      <c r="M9" s="33"/>
-      <c r="N9" s="33"/>
+        <v>630</v>
+      </c>
+      <c r="K9" s="33" t="s">
+        <v>845</v>
+      </c>
+      <c r="L9" s="36" t="n">
+        <v>46320</v>
+      </c>
+      <c r="M9" s="33" t="s">
+        <v>846</v>
+      </c>
+      <c r="N9" s="33" t="s">
+        <v>847</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="31" t="s">
-        <v>828</v>
+        <v>848</v>
       </c>
       <c r="B10" s="31" t="s">
         <v>5</v>
       </c>
       <c r="C10" s="31" t="s">
-        <v>829</v>
+        <v>849</v>
       </c>
       <c r="D10" s="31" t="s">
-        <v>830</v>
+        <v>850</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="F10" s="40" t="n">
         <v>5</v>
       </c>
       <c r="G10" s="31" t="s">
-        <v>812</v>
+        <v>829</v>
       </c>
       <c r="H10" s="41"/>
       <c r="I10" s="31" t="str">
@@ -14822,7 +14999,7 @@
         <v>PENDING</v>
       </c>
       <c r="J10" s="31" t="s">
-        <v>831</v>
+        <v>851</v>
       </c>
       <c r="K10" s="33"/>
       <c r="L10" s="36"/>
@@ -14831,25 +15008,25 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="31" t="s">
-        <v>832</v>
+        <v>852</v>
       </c>
       <c r="B11" s="31" t="s">
         <v>5</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>829</v>
+        <v>849</v>
       </c>
       <c r="D11" s="31" t="s">
-        <v>833</v>
+        <v>853</v>
       </c>
       <c r="E11" s="31" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="F11" s="40" t="n">
         <v>30</v>
       </c>
       <c r="G11" s="31" t="s">
-        <v>812</v>
+        <v>829</v>
       </c>
       <c r="H11" s="41"/>
       <c r="I11" s="31" t="str">
@@ -14857,7 +15034,7 @@
         <v>PENDING</v>
       </c>
       <c r="J11" s="31" t="s">
-        <v>831</v>
+        <v>851</v>
       </c>
       <c r="K11" s="33"/>
       <c r="L11" s="36"/>
@@ -14866,25 +15043,25 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="31" t="s">
-        <v>834</v>
+        <v>854</v>
       </c>
       <c r="B12" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>835</v>
+        <v>855</v>
       </c>
       <c r="D12" s="31" t="s">
-        <v>836</v>
+        <v>856</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>804</v>
+        <v>821</v>
       </c>
       <c r="F12" s="40" t="n">
         <v>10000</v>
       </c>
       <c r="G12" s="31" t="s">
-        <v>837</v>
+        <v>857</v>
       </c>
       <c r="H12" s="41"/>
       <c r="I12" s="31" t="str">
@@ -14901,7 +15078,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="31" t="s">
-        <v>838</v>
+        <v>858</v>
       </c>
       <c r="B13" s="31" t="s">
         <v>7</v>
@@ -14910,16 +15087,16 @@
         <v>42</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>839</v>
+        <v>859</v>
       </c>
       <c r="E13" s="31" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="F13" s="40" t="n">
         <v>25</v>
       </c>
       <c r="G13" s="31" t="s">
-        <v>798</v>
+        <v>815</v>
       </c>
       <c r="H13" s="41"/>
       <c r="I13" s="31" t="str">
@@ -14936,7 +15113,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="31" t="s">
-        <v>840</v>
+        <v>860</v>
       </c>
       <c r="B14" s="31" t="s">
         <v>7</v>
@@ -14945,16 +15122,16 @@
         <v>42</v>
       </c>
       <c r="D14" s="31" t="s">
-        <v>841</v>
+        <v>861</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="F14" s="40" t="n">
         <v>50</v>
       </c>
       <c r="G14" s="31" t="s">
-        <v>798</v>
+        <v>815</v>
       </c>
       <c r="H14" s="41"/>
       <c r="I14" s="31" t="str">
@@ -14971,25 +15148,25 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="31" t="s">
-        <v>842</v>
+        <v>862</v>
       </c>
       <c r="B15" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>843</v>
+        <v>863</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>844</v>
+        <v>864</v>
       </c>
       <c r="E15" s="31" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="F15" s="38" t="n">
         <v>0.001</v>
       </c>
       <c r="G15" s="31" t="s">
-        <v>805</v>
+        <v>822</v>
       </c>
       <c r="H15" s="39"/>
       <c r="I15" s="31" t="str">
@@ -15006,25 +15183,25 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="31" t="s">
-        <v>845</v>
+        <v>865</v>
       </c>
       <c r="B16" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C16" s="31" t="s">
-        <v>846</v>
+        <v>866</v>
       </c>
       <c r="D16" s="31" t="s">
-        <v>847</v>
+        <v>867</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="F16" s="40" t="n">
         <v>0</v>
       </c>
       <c r="G16" s="31" t="s">
-        <v>848</v>
+        <v>868</v>
       </c>
       <c r="H16" s="41"/>
       <c r="I16" s="31" t="str">
@@ -15032,7 +15209,7 @@
         <v>PENDING</v>
       </c>
       <c r="J16" s="31" t="s">
-        <v>737</v>
+        <v>742</v>
       </c>
       <c r="K16" s="33"/>
       <c r="L16" s="36"/>
@@ -15041,25 +15218,25 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="31" t="s">
-        <v>849</v>
+        <v>869</v>
       </c>
       <c r="B17" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C17" s="31" t="s">
-        <v>846</v>
+        <v>866</v>
       </c>
       <c r="D17" s="31" t="s">
-        <v>850</v>
+        <v>870</v>
       </c>
       <c r="E17" s="31" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="F17" s="40" t="n">
         <v>0</v>
       </c>
       <c r="G17" s="31" t="s">
-        <v>827</v>
+        <v>844</v>
       </c>
       <c r="H17" s="41"/>
       <c r="I17" s="31" t="str">
@@ -15067,7 +15244,7 @@
         <v>PENDING</v>
       </c>
       <c r="J17" s="31" t="s">
-        <v>851</v>
+        <v>871</v>
       </c>
       <c r="K17" s="33"/>
       <c r="L17" s="36"/>
@@ -15076,25 +15253,25 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="31" t="s">
-        <v>852</v>
+        <v>872</v>
       </c>
       <c r="B18" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C18" s="31" t="s">
-        <v>853</v>
+        <v>873</v>
       </c>
       <c r="D18" s="31" t="s">
-        <v>854</v>
+        <v>874</v>
       </c>
       <c r="E18" s="31" t="s">
-        <v>804</v>
+        <v>821</v>
       </c>
       <c r="F18" s="38" t="n">
         <v>0.999</v>
       </c>
       <c r="G18" s="31" t="s">
-        <v>805</v>
+        <v>822</v>
       </c>
       <c r="H18" s="39"/>
       <c r="I18" s="31" t="str">
@@ -15102,7 +15279,7 @@
         <v>PENDING</v>
       </c>
       <c r="J18" s="31" t="s">
-        <v>855</v>
+        <v>875</v>
       </c>
       <c r="K18" s="33"/>
       <c r="L18" s="36"/>
@@ -15111,7 +15288,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="31" t="s">
-        <v>856</v>
+        <v>876</v>
       </c>
       <c r="B19" s="31" t="s">
         <v>7</v>
@@ -15120,16 +15297,16 @@
         <v>42</v>
       </c>
       <c r="D19" s="31" t="s">
-        <v>857</v>
+        <v>877</v>
       </c>
       <c r="E19" s="31" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="F19" s="40" t="n">
         <v>2</v>
       </c>
       <c r="G19" s="31" t="s">
-        <v>858</v>
+        <v>878</v>
       </c>
       <c r="H19" s="41"/>
       <c r="I19" s="31" t="str">
@@ -15137,7 +15314,7 @@
         <v>PENDING</v>
       </c>
       <c r="J19" s="31" t="s">
-        <v>859</v>
+        <v>879</v>
       </c>
       <c r="K19" s="33"/>
       <c r="L19" s="36"/>
@@ -15146,25 +15323,25 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="31" t="s">
-        <v>860</v>
+        <v>880</v>
       </c>
       <c r="B20" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C20" s="31" t="s">
-        <v>861</v>
+        <v>881</v>
       </c>
       <c r="D20" s="31" t="s">
-        <v>862</v>
+        <v>882</v>
       </c>
       <c r="E20" s="31" t="s">
-        <v>797</v>
+        <v>814</v>
       </c>
       <c r="F20" s="40" t="n">
         <v>15</v>
       </c>
       <c r="G20" s="31" t="s">
-        <v>812</v>
+        <v>829</v>
       </c>
       <c r="H20" s="41"/>
       <c r="I20" s="31" t="str">
@@ -15172,7 +15349,7 @@
         <v>PENDING</v>
       </c>
       <c r="J20" s="31" t="s">
-        <v>863</v>
+        <v>883</v>
       </c>
       <c r="K20" s="33"/>
       <c r="L20" s="36"/>
@@ -15181,25 +15358,25 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="31" t="s">
-        <v>864</v>
+        <v>884</v>
       </c>
       <c r="B21" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C21" s="31" t="s">
-        <v>865</v>
+        <v>885</v>
       </c>
       <c r="D21" s="31" t="s">
-        <v>866</v>
+        <v>886</v>
       </c>
       <c r="E21" s="31" t="s">
-        <v>804</v>
+        <v>821</v>
       </c>
       <c r="F21" s="38" t="n">
         <v>0.9</v>
       </c>
       <c r="G21" s="31" t="s">
-        <v>805</v>
+        <v>822</v>
       </c>
       <c r="H21" s="39"/>
       <c r="I21" s="31" t="str">
@@ -15216,25 +15393,25 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="31" t="s">
-        <v>867</v>
+        <v>887</v>
       </c>
       <c r="B22" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C22" s="31" t="s">
-        <v>865</v>
+        <v>885</v>
       </c>
       <c r="D22" s="31" t="s">
-        <v>868</v>
+        <v>888</v>
       </c>
       <c r="E22" s="31" t="s">
-        <v>804</v>
+        <v>821</v>
       </c>
       <c r="F22" s="38" t="n">
         <v>0.75</v>
       </c>
       <c r="G22" s="31" t="s">
-        <v>805</v>
+        <v>822</v>
       </c>
       <c r="H22" s="39"/>
       <c r="I22" s="31" t="str">
@@ -15242,7 +15419,7 @@
         <v>PENDING</v>
       </c>
       <c r="J22" s="31" t="s">
-        <v>695</v>
+        <v>700</v>
       </c>
       <c r="K22" s="33"/>
       <c r="L22" s="36"/>
@@ -15251,25 +15428,25 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="31" t="s">
-        <v>869</v>
+        <v>889</v>
       </c>
       <c r="B23" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="31" t="s">
-        <v>802</v>
+        <v>819</v>
       </c>
       <c r="D23" s="31" t="s">
-        <v>870</v>
+        <v>890</v>
       </c>
       <c r="E23" s="31" t="s">
-        <v>804</v>
+        <v>821</v>
       </c>
       <c r="F23" s="38" t="n">
         <v>0.9995</v>
       </c>
       <c r="G23" s="31" t="s">
-        <v>805</v>
+        <v>822</v>
       </c>
       <c r="H23" s="39"/>
       <c r="I23" s="31" t="str">
@@ -15277,7 +15454,7 @@
         <v>PENDING</v>
       </c>
       <c r="J23" s="31" t="s">
-        <v>806</v>
+        <v>823</v>
       </c>
       <c r="K23" s="33"/>
       <c r="L23" s="36"/>
@@ -15348,7 +15525,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>871</v>
+        <v>891</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>140</v>
@@ -15363,55 +15540,55 @@
         <v>589</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>872</v>
+        <v>892</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>873</v>
+        <v>893</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>874</v>
+        <v>894</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>875</v>
+        <v>895</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>876</v>
+        <v>896</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>877</v>
+        <v>897</v>
       </c>
       <c r="L1" s="13" t="s">
-        <v>878</v>
+        <v>898</v>
       </c>
       <c r="M1" s="13" t="s">
-        <v>879</v>
+        <v>899</v>
       </c>
       <c r="N1" s="13" t="s">
-        <v>880</v>
+        <v>900</v>
       </c>
       <c r="O1" s="13" t="s">
-        <v>881</v>
+        <v>901</v>
       </c>
       <c r="P1" s="13" t="s">
-        <v>882</v>
+        <v>902</v>
       </c>
       <c r="Q1" s="13" t="s">
-        <v>883</v>
+        <v>903</v>
       </c>
       <c r="R1" s="13" t="s">
-        <v>884</v>
+        <v>904</v>
       </c>
       <c r="S1" s="13" t="s">
-        <v>885</v>
+        <v>905</v>
       </c>
       <c r="T1" s="13" t="s">
-        <v>791</v>
+        <v>808</v>
       </c>
       <c r="U1" s="13" t="s">
-        <v>794</v>
+        <v>811</v>
       </c>
       <c r="V1" s="13" t="s">
-        <v>886</v>
+        <v>906</v>
       </c>
       <c r="W1" s="13" t="s">
         <v>594</v>
@@ -15419,7 +15596,7 @@
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="s">
-        <v>799</v>
+        <v>816</v>
       </c>
       <c r="B2" s="28" t="s">
         <v>157</v>
@@ -15428,13 +15605,13 @@
         <v>114</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>887</v>
+        <v>907</v>
       </c>
       <c r="E2" s="28" t="s">
         <v>470</v>
       </c>
       <c r="F2" s="28" t="s">
-        <v>888</v>
+        <v>908</v>
       </c>
       <c r="G2" s="28" t="n">
         <v>30</v>
@@ -15484,15 +15661,15 @@
         <v>46338</v>
       </c>
       <c r="V2" s="28" t="s">
-        <v>889</v>
+        <v>909</v>
       </c>
       <c r="W2" s="28" t="s">
-        <v>800</v>
+        <v>817</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="31" t="s">
-        <v>890</v>
+        <v>910</v>
       </c>
       <c r="B3" s="31" t="s">
         <v>5</v>
@@ -15501,13 +15678,13 @@
         <v>114</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>891</v>
+        <v>911</v>
       </c>
       <c r="E3" s="31" t="s">
         <v>372</v>
       </c>
       <c r="F3" s="31" t="s">
-        <v>892</v>
+        <v>912</v>
       </c>
       <c r="G3" s="31" t="n">
         <v>15</v>
@@ -15543,7 +15720,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>893</v>
+        <v>913</v>
       </c>
       <c r="B4" s="31" t="s">
         <v>5</v>
@@ -15552,13 +15729,13 @@
         <v>116</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>894</v>
+        <v>914</v>
       </c>
       <c r="E4" s="31" t="s">
         <v>372</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>888</v>
+        <v>908</v>
       </c>
       <c r="G4" s="31" t="n">
         <v>5</v>
@@ -15594,7 +15771,7 @@
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>895</v>
+        <v>915</v>
       </c>
       <c r="B5" s="31" t="s">
         <v>7</v>
@@ -15603,13 +15780,13 @@
         <v>114</v>
       </c>
       <c r="D5" s="31" t="s">
-        <v>896</v>
+        <v>916</v>
       </c>
       <c r="E5" s="31" t="s">
         <v>470</v>
       </c>
       <c r="F5" s="31" t="s">
-        <v>897</v>
+        <v>917</v>
       </c>
       <c r="G5" s="31" t="n">
         <v>30</v>
@@ -15645,7 +15822,7 @@
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="31" t="s">
-        <v>898</v>
+        <v>918</v>
       </c>
       <c r="B6" s="31" t="s">
         <v>7</v>
@@ -15654,13 +15831,13 @@
         <v>115</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>899</v>
+        <v>919</v>
       </c>
       <c r="E6" s="31" t="s">
         <v>470</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>888</v>
+        <v>908</v>
       </c>
       <c r="G6" s="31" t="n">
         <v>30</v>
@@ -15696,7 +15873,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="31" t="s">
-        <v>900</v>
+        <v>920</v>
       </c>
       <c r="B7" s="31" t="s">
         <v>7</v>
@@ -15705,13 +15882,13 @@
         <v>116</v>
       </c>
       <c r="D7" s="31" t="s">
-        <v>901</v>
+        <v>921</v>
       </c>
       <c r="E7" s="31" t="s">
         <v>470</v>
       </c>
       <c r="F7" s="31" t="s">
-        <v>888</v>
+        <v>908</v>
       </c>
       <c r="G7" s="31" t="n">
         <v>5</v>
@@ -15747,7 +15924,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="31" t="s">
-        <v>902</v>
+        <v>922</v>
       </c>
       <c r="B8" s="31" t="s">
         <v>7</v>
@@ -15756,13 +15933,13 @@
         <v>117</v>
       </c>
       <c r="D8" s="31" t="s">
-        <v>903</v>
+        <v>923</v>
       </c>
       <c r="E8" s="31" t="s">
         <v>483</v>
       </c>
       <c r="F8" s="31" t="s">
-        <v>888</v>
+        <v>908</v>
       </c>
       <c r="G8" s="31" t="n">
         <v>480</v>
@@ -15798,7 +15975,7 @@
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="31" t="s">
-        <v>904</v>
+        <v>924</v>
       </c>
       <c r="B9" s="31" t="s">
         <v>7</v>
@@ -15807,13 +15984,13 @@
         <v>118</v>
       </c>
       <c r="D9" s="31" t="s">
-        <v>905</v>
+        <v>925</v>
       </c>
       <c r="E9" s="31" t="s">
         <v>470</v>
       </c>
       <c r="F9" s="31" t="s">
-        <v>888</v>
+        <v>908</v>
       </c>
       <c r="G9" s="31" t="n">
         <v>30</v>
@@ -15849,7 +16026,7 @@
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="31" t="s">
-        <v>906</v>
+        <v>926</v>
       </c>
       <c r="B10" s="31" t="s">
         <v>7</v>
@@ -15858,13 +16035,13 @@
         <v>119</v>
       </c>
       <c r="D10" s="31" t="s">
-        <v>907</v>
+        <v>927</v>
       </c>
       <c r="E10" s="31" t="s">
-        <v>785</v>
+        <v>790</v>
       </c>
       <c r="F10" s="31" t="s">
-        <v>888</v>
+        <v>908</v>
       </c>
       <c r="G10" s="31" t="n">
         <v>15</v>
@@ -15951,43 +16128,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="13" t="s">
-        <v>908</v>
+        <v>928</v>
       </c>
       <c r="B1" s="13" t="s">
         <v>140</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>909</v>
+        <v>929</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>910</v>
+        <v>930</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>911</v>
+        <v>931</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>912</v>
+        <v>932</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>913</v>
+        <v>933</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>914</v>
+        <v>934</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>915</v>
+        <v>935</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>916</v>
+        <v>936</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>917</v>
+        <v>937</v>
       </c>
       <c r="L1" s="13" t="s">
-        <v>794</v>
+        <v>811</v>
       </c>
       <c r="M1" s="13" t="s">
-        <v>791</v>
+        <v>808</v>
       </c>
       <c r="N1" s="13" t="s">
         <v>594</v>
@@ -15995,28 +16172,28 @@
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="s">
-        <v>918</v>
+        <v>938</v>
       </c>
       <c r="B2" s="28" t="s">
         <v>157</v>
       </c>
       <c r="C2" s="28" t="s">
-        <v>919</v>
+        <v>939</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>920</v>
+        <v>940</v>
       </c>
       <c r="E2" s="28" t="s">
-        <v>921</v>
+        <v>941</v>
       </c>
       <c r="F2" s="28" t="s">
-        <v>765</v>
+        <v>770</v>
       </c>
       <c r="G2" s="28" t="s">
-        <v>922</v>
+        <v>942</v>
       </c>
       <c r="H2" s="28" t="s">
-        <v>923</v>
+        <v>943</v>
       </c>
       <c r="I2" s="28" t="n">
         <v>12</v>
@@ -16025,7 +16202,7 @@
         <v>30</v>
       </c>
       <c r="K2" s="28" t="s">
-        <v>924</v>
+        <v>944</v>
       </c>
       <c r="L2" s="29" t="n">
         <v>46340</v>
@@ -16035,30 +16212,30 @@
         <v>PASS</v>
       </c>
       <c r="N2" s="28" t="s">
-        <v>925</v>
+        <v>945</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="31" t="s">
-        <v>926</v>
+        <v>946</v>
       </c>
       <c r="B3" s="31" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>927</v>
+        <v>947</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>928</v>
+        <v>948</v>
       </c>
       <c r="E3" s="31" t="s">
-        <v>929</v>
+        <v>949</v>
       </c>
       <c r="F3" s="31" t="s">
-        <v>930</v>
+        <v>950</v>
       </c>
       <c r="G3" s="31" t="s">
-        <v>931</v>
+        <v>951</v>
       </c>
       <c r="H3" s="33"/>
       <c r="I3" s="33"/>
@@ -16075,25 +16252,25 @@
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
-        <v>932</v>
+        <v>952</v>
       </c>
       <c r="B4" s="31" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>933</v>
+        <v>953</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>934</v>
+        <v>954</v>
       </c>
       <c r="E4" s="31" t="s">
-        <v>935</v>
+        <v>955</v>
       </c>
       <c r="F4" s="31" t="s">
-        <v>936</v>
+        <v>956</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>937</v>
+        <v>957</v>
       </c>
       <c r="H4" s="33"/>
       <c r="I4" s="33"/>
@@ -16110,25 +16287,25 @@
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
-        <v>938</v>
+        <v>958</v>
       </c>
       <c r="B5" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C5" s="31" t="s">
-        <v>919</v>
+        <v>939</v>
       </c>
       <c r="D5" s="31" t="s">
-        <v>939</v>
+        <v>959</v>
       </c>
       <c r="E5" s="31" t="s">
-        <v>940</v>
+        <v>960</v>
       </c>
       <c r="F5" s="31" t="s">
-        <v>765</v>
+        <v>770</v>
       </c>
       <c r="G5" s="31" t="s">
-        <v>941</v>
+        <v>961</v>
       </c>
       <c r="H5" s="33"/>
       <c r="I5" s="33"/>
@@ -16145,25 +16322,25 @@
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="31" t="s">
-        <v>942</v>
+        <v>962</v>
       </c>
       <c r="B6" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>943</v>
+        <v>963</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>944</v>
+        <v>964</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>945</v>
+        <v>965</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>749</v>
+        <v>754</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>946</v>
+        <v>966</v>
       </c>
       <c r="H6" s="33"/>
       <c r="I6" s="33"/>
@@ -16180,25 +16357,25 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="31" t="s">
-        <v>947</v>
+        <v>967</v>
       </c>
       <c r="B7" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="31" t="s">
-        <v>948</v>
+        <v>968</v>
       </c>
       <c r="D7" s="31" t="s">
-        <v>949</v>
+        <v>969</v>
       </c>
       <c r="E7" s="31" t="s">
-        <v>950</v>
+        <v>970</v>
       </c>
       <c r="F7" s="31" t="s">
-        <v>951</v>
+        <v>971</v>
       </c>
       <c r="G7" s="31" t="s">
-        <v>952</v>
+        <v>972</v>
       </c>
       <c r="H7" s="33"/>
       <c r="I7" s="33"/>
@@ -16215,25 +16392,25 @@
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="31" t="s">
-        <v>953</v>
+        <v>973</v>
       </c>
       <c r="B8" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="31" t="s">
-        <v>954</v>
+        <v>974</v>
       </c>
       <c r="D8" s="31" t="s">
-        <v>955</v>
+        <v>975</v>
       </c>
       <c r="E8" s="31" t="s">
-        <v>956</v>
+        <v>976</v>
       </c>
       <c r="F8" s="31" t="s">
-        <v>957</v>
+        <v>977</v>
       </c>
       <c r="G8" s="31" t="s">
-        <v>958</v>
+        <v>978</v>
       </c>
       <c r="H8" s="33"/>
       <c r="I8" s="33"/>
@@ -16250,25 +16427,25 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="31" t="s">
-        <v>959</v>
+        <v>979</v>
       </c>
       <c r="B9" s="31" t="s">
         <v>7</v>
       </c>
       <c r="C9" s="31" t="s">
-        <v>960</v>
+        <v>980</v>
       </c>
       <c r="D9" s="31" t="s">
-        <v>961</v>
+        <v>981</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>962</v>
+        <v>982</v>
       </c>
       <c r="F9" s="31" t="s">
         <v>109</v>
       </c>
       <c r="G9" s="31" t="s">
-        <v>963</v>
+        <v>983</v>
       </c>
       <c r="H9" s="33"/>
       <c r="I9" s="33"/>
@@ -16341,37 +16518,37 @@
         <v>140</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>964</v>
+        <v>984</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>965</v>
+        <v>985</v>
       </c>
       <c r="D1" s="13" t="s">
         <v>589</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>966</v>
+        <v>986</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>967</v>
+        <v>987</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>968</v>
+        <v>988</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>969</v>
+        <v>989</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>970</v>
+        <v>990</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>971</v>
+        <v>991</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>791</v>
+        <v>808</v>
       </c>
       <c r="L1" s="13" t="s">
-        <v>794</v>
+        <v>811</v>
       </c>
       <c r="M1" s="13" t="s">
         <v>594</v>
@@ -16382,13 +16559,13 @@
         <v>157</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>972</v>
+        <v>992</v>
       </c>
       <c r="C2" s="28" t="s">
-        <v>973</v>
+        <v>993</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>974</v>
+        <v>994</v>
       </c>
       <c r="E2" s="30" t="n">
         <v>0.93</v>
@@ -16416,7 +16593,7 @@
         <v>46346</v>
       </c>
       <c r="M2" s="28" t="s">
-        <v>975</v>
+        <v>995</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16424,17 +16601,23 @@
         <v>5</v>
       </c>
       <c r="B3" s="31" t="s">
-        <v>976</v>
+        <v>996</v>
       </c>
       <c r="C3" s="31" t="s">
-        <v>973</v>
+        <v>993</v>
       </c>
       <c r="D3" s="31" t="s">
-        <v>974</v>
-      </c>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
+        <v>994</v>
+      </c>
+      <c r="E3" s="34" t="n">
+        <v>0.974</v>
+      </c>
+      <c r="F3" s="34" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="G3" s="34" t="n">
+        <v>0.88</v>
+      </c>
       <c r="H3" s="35" t="n">
         <v>0.9</v>
       </c>
@@ -16446,27 +16629,37 @@
       </c>
       <c r="K3" s="31" t="str">
         <f aca="false">IF(OR(E3="",F3="",G3=""),"PENDING",IF(AND(E3&gt;=H3,F3&gt;=I3,G3&gt;=J3),"PASS","FAIL"))</f>
-        <v>PENDING</v>
-      </c>
-      <c r="L3" s="36"/>
-      <c r="M3" s="33"/>
+        <v>PASS</v>
+      </c>
+      <c r="L3" s="36" t="n">
+        <v>46320</v>
+      </c>
+      <c r="M3" s="33" t="s">
+        <v>997</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="31" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="31" t="s">
-        <v>977</v>
+        <v>998</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>973</v>
+        <v>993</v>
       </c>
       <c r="D4" s="31" t="s">
-        <v>974</v>
-      </c>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
+        <v>994</v>
+      </c>
+      <c r="E4" s="34" t="n">
+        <v>0.997</v>
+      </c>
+      <c r="F4" s="34" t="n">
+        <v>0.936</v>
+      </c>
+      <c r="G4" s="34" t="n">
+        <v>0.943</v>
+      </c>
       <c r="H4" s="35" t="n">
         <v>0.9</v>
       </c>
@@ -16478,23 +16671,27 @@
       </c>
       <c r="K4" s="31" t="str">
         <f aca="false">IF(OR(E4="",F4="",G4=""),"PENDING",IF(AND(E4&gt;=H4,F4&gt;=I4,G4&gt;=J4),"PASS","FAIL"))</f>
-        <v>PENDING</v>
-      </c>
-      <c r="L4" s="36"/>
-      <c r="M4" s="33"/>
+        <v>PASS</v>
+      </c>
+      <c r="L4" s="36" t="n">
+        <v>46320</v>
+      </c>
+      <c r="M4" s="33" t="s">
+        <v>997</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="31" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="31" t="s">
-        <v>972</v>
+        <v>992</v>
       </c>
       <c r="C5" s="31" t="s">
-        <v>973</v>
+        <v>993</v>
       </c>
       <c r="D5" s="31" t="s">
-        <v>974</v>
+        <v>994</v>
       </c>
       <c r="E5" s="34"/>
       <c r="F5" s="34"/>
@@ -16520,13 +16717,13 @@
         <v>7</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>978</v>
+        <v>999</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>973</v>
+        <v>993</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>974</v>
+        <v>994</v>
       </c>
       <c r="E6" s="34"/>
       <c r="F6" s="34"/>
@@ -16552,13 +16749,13 @@
         <v>7</v>
       </c>
       <c r="B7" s="31" t="s">
-        <v>979</v>
+        <v>1000</v>
       </c>
       <c r="C7" s="31" t="s">
-        <v>973</v>
+        <v>993</v>
       </c>
       <c r="D7" s="31" t="s">
-        <v>974</v>
+        <v>994</v>
       </c>
       <c r="E7" s="34"/>
       <c r="F7" s="34"/>
@@ -16584,13 +16781,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="31" t="s">
-        <v>980</v>
+        <v>1001</v>
       </c>
       <c r="C8" s="31" t="s">
-        <v>973</v>
+        <v>993</v>
       </c>
       <c r="D8" s="31" t="s">
-        <v>974</v>
+        <v>994</v>
       </c>
       <c r="E8" s="34"/>
       <c r="F8" s="34"/>

</xml_diff>

<commit_message>
chore: correct the record for TC-PLT-005 and coverage; evidence addendum
TC-PLT-005 had been marked passing while the CodeQL gate could not fail and
main had five open high alerts; it now cites the run after they were fixed
and triaged (0 open). Coverage rows cite CI runs. The evidence gains a
section on what the review found.
</commit_message>
<xml_diff>
--- a/tracker/Meterbook_Tracker.xlsx
+++ b/tracker/Meterbook_Tracker.xlsx
@@ -163,7 +163,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1923" uniqueCount="1025">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1923" uniqueCount="1026">
   <si>
     <t xml:space="preserve">Meterbook — Plan, Test &amp; Reliability Tracker</t>
   </si>
@@ -2043,10 +2043,10 @@
     <t xml:space="preserve">0 high/critical findings</t>
   </si>
   <si>
-    <t xml:space="preserve">CodeQL (security-extended; Java, Python, Actions) on every PR, main and weekly: 0 high/critical (a finding &gt;= 7.0 fails the run); Semgrep p/default on every change: 0 errors/warnings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://github.com/mhrj7/meterbook/actions/runs/40122321805</t>
+    <t xml:space="preserve">0 open high/critical on main (code scanning). The first gate read severities from the wrong SARIF field and could not fail; fixed, it found 5 high: 2 user-controlled-bypass fixed in code, 3 CSRF-disabled excluded with reason (stateless, header-only credentials; NoAmbientCredentialsTest guards it). Semgrep p/default: 0.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/mhrj7/meterbook/actions/runs/40143497435</t>
   </si>
   <si>
     <t xml:space="preserve">TC-PLT-006</t>
@@ -3156,10 +3156,13 @@
     <t xml:space="preserve">identity</t>
   </si>
   <si>
-    <t xml:space="preserve">https://github.com/mhrj7/meterbook/actions/runs/40120018649</t>
+    <t xml:space="preserve">line/branch: https://github.com/mhrj7/meterbook/actions/runs/40143043993 ; mutation: https://github.com/mhrj7/meterbook/actions/runs/40120018649</t>
   </si>
   <si>
     <t xml:space="preserve">tenancy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">line/branch: local JaCoCo per-package (CI reports the module total); mutation: https://github.com/mhrj7/meterbook/actions/runs/40120018649</t>
   </si>
   <si>
     <t xml:space="preserve">pricing</t>
@@ -4344,54 +4347,54 @@
         <v>140</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>1002</v>
+        <v>1003</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>1003</v>
+        <v>1004</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="F1" s="13" t="s">
         <v>148</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="K1" s="13" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="L1" s="13" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="B2" s="28" t="s">
         <v>157</v>
       </c>
       <c r="C2" s="28" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="E2" s="28" t="s">
         <v>705</v>
       </c>
       <c r="F2" s="28" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="G2" s="29" t="n">
         <v>46336</v>
@@ -4404,10 +4407,10 @@
         <v>1</v>
       </c>
       <c r="J2" s="28" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="K2" s="28" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="L2" s="28" t="s">
         <v>599</v>
@@ -6164,31 +6167,31 @@
         <v>145</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="G1" s="13" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="H1" s="13" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="I1" s="13" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="J1" s="13" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="K1" s="13" t="s">
         <v>594</v>
@@ -8402,7 +8405,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{335289DB-DB61-408A-87EF-B07A376756B3}</x14:id>
+          <x14:id>{BDB670CA-EE6E-40E6-B32A-2428B870B4B9}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8416,7 +8419,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{C979CEB7-F435-4329-AD6E-5EECE5235CCE}</x14:id>
+          <x14:id>{77E8D630-9192-43D1-9C10-5A837F5A5BE4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8430,7 +8433,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{14D6A86A-A5CA-43DB-BABA-C785A5B749CE}</x14:id>
+          <x14:id>{55444862-616B-49CB-9C40-7274D22D20D4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8444,7 +8447,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{86D04ABD-1823-45B5-A3D3-DA6F2BA3C52F}</x14:id>
+          <x14:id>{8E5E5543-2094-41AF-8D1E-3DBC278DD512}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8490,7 +8493,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{335289DB-DB61-408A-87EF-B07A376756B3}">
+          <x14:cfRule type="dataBar" id="{BDB670CA-EE6E-40E6-B32A-2428B870B4B9}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -8505,7 +8508,7 @@
           <xm:sqref>B14:D14</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{C979CEB7-F435-4329-AD6E-5EECE5235CCE}">
+          <x14:cfRule type="dataBar" id="{77E8D630-9192-43D1-9C10-5A837F5A5BE4}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -8520,7 +8523,7 @@
           <xm:sqref>B22:D22</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{14D6A86A-A5CA-43DB-BABA-C785A5B749CE}">
+          <x14:cfRule type="dataBar" id="{55444862-616B-49CB-9C40-7274D22D20D4}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -8535,7 +8538,7 @@
           <xm:sqref>B23:D23</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{86D04ABD-1823-45B5-A3D3-DA6F2BA3C52F}">
+          <x14:cfRule type="dataBar" id="{8E5E5543-2094-41AF-8D1E-3DBC278DD512}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -10718,7 +10721,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{A4B27AF6-B282-44F5-988D-F9DA739DB031}</x14:id>
+          <x14:id>{2013909B-892A-44EC-B5D0-36848A762BE4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10749,7 +10752,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{A4B27AF6-B282-44F5-988D-F9DA739DB031}">
+          <x14:cfRule type="dataBar" id="{2013909B-892A-44EC-B5D0-36848A762BE4}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -14462,7 +14465,7 @@
       <c r="N47" s="33"/>
       <c r="O47" s="33"/>
     </row>
-    <row r="48" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="31" t="s">
         <v>791</v>
       </c>
@@ -14508,7 +14511,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="31" t="s">
         <v>798</v>
       </c>
@@ -16613,7 +16616,7 @@
         <v>0.974</v>
       </c>
       <c r="F3" s="34" t="n">
-        <v>0.867</v>
+        <v>0.868</v>
       </c>
       <c r="G3" s="34" t="n">
         <v>0.88</v>
@@ -16677,7 +16680,7 @@
         <v>46320</v>
       </c>
       <c r="M4" s="33" t="s">
-        <v>997</v>
+        <v>999</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16717,7 +16720,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="C6" s="31" t="s">
         <v>993</v>
@@ -16749,7 +16752,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="31" t="s">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="C7" s="31" t="s">
         <v>993</v>
@@ -16781,7 +16784,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="31" t="s">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="C8" s="31" t="s">
         <v>993</v>

</xml_diff>

<commit_message>
docs: branch protection on main is on; ADR-0003 follow-up done
Pull requests only, required checks ci and the three CodeQL analyses,
enforced for administrators, no force-pushes or deletions. TC-PLT-013 and
TC-PLT-014 promised that a failing check blocks the merge; now it does.
</commit_message>
<xml_diff>
--- a/tracker/Meterbook_Tracker.xlsx
+++ b/tracker/Meterbook_Tracker.xlsx
@@ -2151,7 +2151,7 @@
     <t xml:space="preserve">Linters in CI</t>
   </si>
   <si>
-    <t xml:space="preserve">This repo has Java, Python and shell (no Go or Rust): SpotBugs in ./gradlew check (found and fixed 5 real bugs; any finding fails), ruff and ShellCheck on every change; ci requires the job</t>
+    <t xml:space="preserve">This repo has Java, Python and shell (no Go or Rust): SpotBugs in ./gradlew check (found and fixed 5 real bugs; any finding fails), ruff and ShellCheck on every change; ci requires the job Branch protection on main requires ci, so a lint failure blocks the merge.</t>
   </si>
   <si>
     <t xml:space="preserve">https://github.com/mhrj7/meterbook/actions/runs/40122321801</t>
@@ -2169,7 +2169,7 @@
     <t xml:space="preserve">Codecov</t>
   </si>
   <si>
-    <t xml:space="preserve">JaCoCo gate in ./gradlew check (90% line / 85% branch) fails the Java job and the required ci check; identity at 97.4% / 96.6%</t>
+    <t xml:space="preserve">JaCoCo gate in ./gradlew check (90% line / 85% branch) fails the Java job and the required ci check; identity at 97.4% / 96.6% Branch protection on main requires ci, so a coverage failure blocks the merge (2026-10-25).</t>
   </si>
   <si>
     <t xml:space="preserve">TC-PLT-015</t>
@@ -8405,7 +8405,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BDB670CA-EE6E-40E6-B32A-2428B870B4B9}</x14:id>
+          <x14:id>{E03E5F4B-BE40-4B2A-B3F0-177EFAAB297C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8419,7 +8419,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{77E8D630-9192-43D1-9C10-5A837F5A5BE4}</x14:id>
+          <x14:id>{45AEEDC5-FB80-4B44-9B28-D49494EF7860}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8433,7 +8433,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{55444862-616B-49CB-9C40-7274D22D20D4}</x14:id>
+          <x14:id>{20EA9846-4482-46B1-9566-E020E32FBBCB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8447,7 +8447,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8E5E5543-2094-41AF-8D1E-3DBC278DD512}</x14:id>
+          <x14:id>{A24D5793-7814-4E8F-98D9-9B11BD5E8262}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -8493,7 +8493,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BDB670CA-EE6E-40E6-B32A-2428B870B4B9}">
+          <x14:cfRule type="dataBar" id="{E03E5F4B-BE40-4B2A-B3F0-177EFAAB297C}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -8508,7 +8508,7 @@
           <xm:sqref>B14:D14</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{77E8D630-9192-43D1-9C10-5A837F5A5BE4}">
+          <x14:cfRule type="dataBar" id="{45AEEDC5-FB80-4B44-9B28-D49494EF7860}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -8523,7 +8523,7 @@
           <xm:sqref>B22:D22</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{55444862-616B-49CB-9C40-7274D22D20D4}">
+          <x14:cfRule type="dataBar" id="{20EA9846-4482-46B1-9566-E020E32FBBCB}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -8538,7 +8538,7 @@
           <xm:sqref>B23:D23</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8E5E5543-2094-41AF-8D1E-3DBC278DD512}">
+          <x14:cfRule type="dataBar" id="{A24D5793-7814-4E8F-98D9-9B11BD5E8262}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -10721,7 +10721,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2013909B-892A-44EC-B5D0-36848A762BE4}</x14:id>
+          <x14:id>{D350E4E9-1D9B-46F7-A978-9AF98DD869E0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -10752,7 +10752,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2013909B-892A-44EC-B5D0-36848A762BE4}">
+          <x14:cfRule type="dataBar" id="{D350E4E9-1D9B-46F7-A978-9AF98DD869E0}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -13215,7 +13215,7 @@
         <v>378</v>
       </c>
       <c r="L16" s="36" t="n">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="M16" s="33" t="s">
         <v>668</v>

</xml_diff>